<commit_message>
Correct Thailand Jun 2023 entry date to 24 Jun from stamp validity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MuHAkrVAM6ipkG9EkAQkug
</commit_message>
<xml_diff>
--- a/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
+++ b/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>45102</v>
+        <v>45101</v>
       </c>
       <c r="D14" s="10" t="n">
         <v>45104</v>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="J14" s="9" t="inlineStr">
         <is>
-          <t>Passport p.20-21: Thai VOA stamp (entry day partly legible), Thai departed 27 Jun 2023; India dep. RGI Hyderabad 24 Jun 2023</t>
+          <t>Passport p.20-21: Thai VOA stamp admitted 2? Jun 2023 until 9 Jul 2023 (class TR-15 = 15 days -&gt; 24 Jun); Thai departed 27 Jun 2023; India dep. RGI Hyderabad 24 Jun 2023</t>
         </is>
       </c>
       <c r="K14" s="11" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="L14" s="9" t="inlineStr">
         <is>
-          <t>Entry date approx. (24/25 Jun) - please confirm</t>
+          <t>Day digit smudged; 24 Jun inferred from 15-day limit (9 Jul) + India departure 24 Jun</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Belgium, Netherlands, Switzerland and Italy to Jul 2024 Schengen trip
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MuHAkrVAM6ipkG9EkAQkug
</commit_message>
<xml_diff>
--- a/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
+++ b/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
@@ -19,7 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Method" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Travel Log'!$A$4:$L$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Travel Log'!$A$4:$L$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Access Map'!$A$4:$N$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Yatra Visa Planner'!$A$4:$K$36</definedName>
   </definedNames>
@@ -735,12 +735,12 @@
         </is>
       </c>
       <c r="B14" s="6">
-        <f>COUNTIF('Country Summary'!B5:B13,"&gt;0")</f>
+        <f>COUNTIF('Country Summary'!B5:B16,"&gt;0")</f>
         <v/>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Excludes transit-only (Italy)</t>
+          <t>Includes Schengen countries visited Jul 2024</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="B15" s="6">
-        <f>'Country Summary'!B15</f>
+        <f>'Country Summary'!B18</f>
         <v/>
       </c>
       <c r="C15" t="inlineStr">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="B16" s="6">
-        <f>MAX('Country Summary'!B5:B13)</f>
+        <f>MAX('Country Summary'!B5:B16)</f>
         <v/>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -969,7 +969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="L16" s="9" t="inlineStr">
         <is>
-          <t>Schengen trip ~12 days; other Schengen countries visited not stamped - add from itinerary</t>
+          <t>Schengen trip 15-27 Jul 2024 covering France, Belgium, Netherlands, Switzerland, Italy; France dates = whole-trip window, split per country when known</t>
         </is>
       </c>
     </row>
@@ -1708,32 +1708,28 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="n">
-        <v>45500</v>
-      </c>
-      <c r="D17" s="10" t="n">
-        <v>45500</v>
-      </c>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
       <c r="E17" s="9">
         <f>IF(AND(ISNUMBER(C17),ISNUMBER(D17)),D17-C17+1,"")</f>
         <v/>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>Transit</t>
+          <t>Visit</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>Milan Malpensa (MXP)</t>
+          <t>By road/rail within Schengen (no stamp)</t>
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>Milan Malpensa (MXP) -&gt; London Gatwick</t>
+          <t>By road/rail within Schengen (no stamp)</t>
         </is>
       </c>
       <c r="I17" s="9" t="inlineStr">
@@ -1743,7 +1739,7 @@
       </c>
       <c r="J17" s="9" t="inlineStr">
         <is>
-          <t>Passport p.17: Malpensa stamp 27 Jul 2024</t>
+          <t>Your confirmation (Oct 2026): visited during the 15-27 Jul 2024 Europe trip</t>
         </is>
       </c>
       <c r="K17" s="11" t="inlineStr">
@@ -1753,7 +1749,7 @@
       </c>
       <c r="L17" s="9" t="inlineStr">
         <is>
-          <t>Exit/transit stamp (same day as UK entry)</t>
+          <t>Dates unknown - within 15-27 Jul 2024; add from itinerary</t>
         </is>
       </c>
     </row>
@@ -1763,12 +1759,10 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="n">
-        <v>45500</v>
-      </c>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="n"/>
       <c r="D18" s="10" t="n"/>
       <c r="E18" s="9">
         <f>IF(AND(ISNUMBER(C18),ISNUMBER(D18)),D18-C18+1,"")</f>
@@ -1781,32 +1775,32 @@
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>London Gatwick</t>
+          <t>By road/rail within Schengen (no stamp)</t>
         </is>
       </c>
       <c r="H18" s="9" t="inlineStr">
         <is>
-          <t>(UK does not stamp exit)</t>
+          <t>By road/rail within Schengen (no stamp)</t>
         </is>
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
-          <t>UK Standard Visitor C-visit, multiple, 29 Jun-29 Dec 2024</t>
+          <t>Schengen C visa #1</t>
         </is>
       </c>
       <c r="J18" s="9" t="inlineStr">
         <is>
-          <t>Passport p.23: Gatwick stamp 27 Jul 2024</t>
-        </is>
-      </c>
-      <c r="K18" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>Your confirmation (Oct 2026): visited during the 15-27 Jul 2024 Europe trip</t>
+        </is>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
+        <is>
+          <t>Check</t>
         </is>
       </c>
       <c r="L18" s="9" t="inlineStr">
         <is>
-          <t>Left UK by 01 Aug 2024 (UAE entry)</t>
+          <t>Dates unknown - within 15-27 Jul 2024; add from itinerary</t>
         </is>
       </c>
     </row>
@@ -1816,12 +1810,10 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>UAE</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="n">
-        <v>45505</v>
-      </c>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="n"/>
       <c r="D19" s="10" t="n"/>
       <c r="E19" s="9">
         <f>IF(AND(ISNUMBER(C19),ISNUMBER(D19)),D19-C19+1,"")</f>
@@ -1834,32 +1826,32 @@
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>Dubai Intl (DXB)</t>
+          <t>By road/rail within Schengen (no stamp)</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>(UAE does not stamp exit)</t>
+          <t>By road/rail within Schengen (no stamp)</t>
         </is>
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Visa/entry per stamp (Indian PP)</t>
+          <t>Schengen C visa #1</t>
         </is>
       </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
-          <t>Passport p.10: UAE entry stamp 01 Aug 2024; India arrival RGI Hyderabad 05 Aug 2024</t>
-        </is>
-      </c>
-      <c r="K19" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>Your confirmation (Oct 2026): visited during the 15-27 Jul 2024 Europe trip</t>
+        </is>
+      </c>
+      <c r="K19" s="11" t="inlineStr">
+        <is>
+          <t>Check</t>
         </is>
       </c>
       <c r="L19" s="9" t="inlineStr">
         <is>
-          <t>Stayed up to ~4 days</t>
+          <t>Dates unknown - within 15-27 Jul 2024; add from itinerary</t>
         </is>
       </c>
     </row>
@@ -1869,14 +1861,12 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="n">
-        <v>45904</v>
-      </c>
-      <c r="D20" s="12" t="n">
-        <v>45930</v>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n">
+        <v>45500</v>
       </c>
       <c r="E20" s="9">
         <f>IF(AND(ISNUMBER(C20),ISNUMBER(D20)),D20-C20+1,"")</f>
@@ -1889,39 +1879,200 @@
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
+          <t>By road/rail within Schengen (Rome visited)</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>Milan Malpensa (MXP) -&gt; London Gatwick</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>Schengen C visa #1</t>
+        </is>
+      </c>
+      <c r="J20" s="9" t="inlineStr">
+        <is>
+          <t>Your confirmation (Oct 2026): Rome visited; Passport p.17: Malpensa exit stamp 27 Jul 2024</t>
+        </is>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="L20" s="9" t="inlineStr">
+        <is>
+          <t>Entry date unknown - within 15-27 Jul 2024; departed Schengen from Milan</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>45500</v>
+      </c>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="9">
+        <f>IF(AND(ISNUMBER(C21),ISNUMBER(D21)),D21-C21+1,"")</f>
+        <v/>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Visit</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>London Gatwick</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>(UK does not stamp exit)</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>UK Standard Visitor C-visit, multiple, 29 Jun-29 Dec 2024</t>
+        </is>
+      </c>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>Passport p.23: Gatwick stamp 27 Jul 2024</t>
+        </is>
+      </c>
+      <c r="K21" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="inlineStr">
+        <is>
+          <t>Left UK by 01 Aug 2024 (UAE entry)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="n">
+        <v>45505</v>
+      </c>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="9">
+        <f>IF(AND(ISNUMBER(C22),ISNUMBER(D22)),D22-C22+1,"")</f>
+        <v/>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Visit</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>Dubai Intl (DXB)</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>(UAE does not stamp exit)</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Visa/entry per stamp (Indian PP)</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>Passport p.10: UAE entry stamp 01 Aug 2024; India arrival RGI Hyderabad 05 Aug 2024</t>
+        </is>
+      </c>
+      <c r="K22" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>Stayed up to ~4 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="n">
+        <v>45904</v>
+      </c>
+      <c r="D23" s="12" t="n">
+        <v>45930</v>
+      </c>
+      <c r="E23" s="9">
+        <f>IF(AND(ISNUMBER(C23),ISNUMBER(D23)),D23-C23+1,"")</f>
+        <v/>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Visit</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
           <t>USA (CBP admitted 04 Sep 2025)</t>
         </is>
       </c>
-      <c r="H20" s="9" t="inlineStr">
+      <c r="H23" s="9" t="inlineStr">
         <is>
           <t>USA -&gt; Mumbai</t>
         </is>
       </c>
-      <c r="I20" s="9" t="inlineStr">
+      <c r="I23" s="9" t="inlineStr">
         <is>
           <t>B1/B2 10-yr visa (admitted until 03 Mar 2026)</t>
         </is>
       </c>
-      <c r="J20" s="9" t="inlineStr">
+      <c r="J23" s="9" t="inlineStr">
         <is>
           <t>Passport p.26 + p.10: India dep. New Delhi 03 Sep 2025; CBP stamp 04 Sep 2025; India arrival Mumbai 30 Sep 2025</t>
         </is>
       </c>
-      <c r="K20" s="9" t="inlineStr">
+      <c r="K23" s="9" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="L20" s="9" t="inlineStr">
+      <c r="L23" s="9" t="inlineStr">
         <is>
           <t>First use of US visa</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L80"/>
+  <autoFilter ref="A4:L83"/>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Visit,Transit"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1936,7 +2087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1996,280 +2147,364 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="B5" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$80,A5,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A5,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>IFERROR(_xlfn.MINIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A5),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A5,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A5,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>IFERROR(_xlfn.MAXIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A5),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A5,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A5,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E5" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$80,'Travel Log'!$B$5:$B$80,A5,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A5,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>e-Visa (valid 27 Jun-26 Jul 2023); e-Visa (valid to 07 Mar 2023)</t>
+          <t>Schengen C visa #1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="B6" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$80,A6,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A6,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>IFERROR(_xlfn.MINIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A6),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A6,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A6,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>IFERROR(_xlfn.MAXIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A6),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A6,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A6,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$80,'Travel Log'!$B$5:$B$80,A6,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A6,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Schengen C visa #1 (France-issued, Pondicherry)</t>
+          <t>e-Visa (valid 27 Jun-26 Jul 2023); e-Visa (valid to 07 Mar 2023)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>France</t>
         </is>
       </c>
       <c r="B7" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$80,A7,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A7,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>IFERROR(_xlfn.MINIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A7),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A7,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A7,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>IFERROR(_xlfn.MAXIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A7),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A7,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A7,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E7" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$80,'Travel Log'!$B$5:$B$80,A7,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A7,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Schengen C visa #1</t>
+          <t>Schengen C visa #1 (France-issued, Pondicherry)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Nepal</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B8" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$80,A8,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A8,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>IFERROR(_xlfn.MINIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A8),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A8,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A8,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>IFERROR(_xlfn.MAXIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A8),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A8,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A8,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$80,'Travel Log'!$B$5:$B$80,A8,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A8,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>No visa needed; No visa needed (Indian PP)</t>
+          <t>Schengen C visa #1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Sri Lanka</t>
+          <t>Nepal</t>
         </is>
       </c>
       <c r="B9" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$80,A9,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A9,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>IFERROR(_xlfn.MINIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A9),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A9,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A9,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>IFERROR(_xlfn.MAXIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A9),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A9,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A9,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E9" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$80,'Travel Log'!$B$5:$B$80,A9,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A9,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>ETA 30-day, 1st visit (exp 16/01/2020); ETA 30-day, 1st visit (exp 23/02/2022); ETA 30-day, 1st visit (exp 28/10/2019)</t>
+          <t>No visa needed; No visa needed (Indian PP)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="B10" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$80,A10,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A10,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>IFERROR(_xlfn.MINIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A10),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A10,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A10,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>IFERROR(_xlfn.MAXIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A10),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A10,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A10,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$80,'Travel Log'!$B$5:$B$80,A10,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A10,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Visa on Arrival; Visa on Arrival (30 days)</t>
+          <t>Schengen C visa #1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>Sri Lanka</t>
         </is>
       </c>
       <c r="B11" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$80,A11,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A11,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>IFERROR(_xlfn.MINIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A11),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A11,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A11,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>IFERROR(_xlfn.MAXIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A11),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A11,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A11,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E11" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$80,'Travel Log'!$B$5:$B$80,A11,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A11,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Visa/entry per stamp (Indian PP)</t>
+          <t>ETA 30-day, 1st visit (exp 16/01/2020); ETA 30-day, 1st visit (exp 23/02/2022); ETA 30-day, 1st visit (exp 28/10/2019)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="B12" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$80,A12,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A12,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="C12" s="12">
-        <f>IFERROR(_xlfn.MINIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A12),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A12,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A12,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D12" s="12">
-        <f>IFERROR(_xlfn.MAXIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A12),"")</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A12,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A12,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$80,'Travel Log'!$B$5:$B$80,A12,'Travel Log'!$F$5:$F$80,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A12,'Travel Log'!$F$5:$F$83,"Visit")</f>
         <v/>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>B1/B2 10-yr visa (admitted until 03 Mar 2026)</t>
+          <t>Schengen C visa #1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="B13" s="9">
+        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A13,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <v/>
+      </c>
+      <c r="C13" s="12">
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A13,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A13,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="D13" s="12">
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A13,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A13,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="E13" s="9">
+        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A13,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <v/>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Visa on Arrival; Visa on Arrival (30 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="B14" s="9">
+        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A14,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <v/>
+      </c>
+      <c r="C14" s="12">
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A14,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A14,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="D14" s="12">
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A14,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A14,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="E14" s="9">
+        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A14,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <v/>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Visa/entry per stamp (Indian PP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="B15" s="9">
+        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A15,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <v/>
+      </c>
+      <c r="C15" s="12">
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A15,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A15,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="D15" s="12">
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A15,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A15,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="E15" s="9">
+        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A15,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <v/>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>B1/B2 10-yr visa (admitted until 03 Mar 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B13" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$80,A13,'Travel Log'!$F$5:$F$80,"Visit")</f>
-        <v/>
-      </c>
-      <c r="C13" s="12">
-        <f>IFERROR(_xlfn.MINIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A13),"")</f>
-        <v/>
-      </c>
-      <c r="D13" s="12">
-        <f>IFERROR(_xlfn.MAXIFS('Travel Log'!$C$5:$C$80,'Travel Log'!$B$5:$B$80,A13),"")</f>
-        <v/>
-      </c>
-      <c r="E13" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$80,'Travel Log'!$B$5:$B$80,A13,'Travel Log'!$F$5:$F$80,"Visit")</f>
-        <v/>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="B16" s="9">
+        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A16,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <v/>
+      </c>
+      <c r="C16" s="12">
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A16,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A16,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="D16" s="12">
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A16,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A16,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="E16" s="9">
+        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A16,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <v/>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>UK Standard Visitor C-visit, multiple, 29 Jun-29 Dec 2024</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B15" s="4">
-        <f>SUM(B5:B13)</f>
-        <v/>
-      </c>
-      <c r="E15" s="4">
-        <f>SUM(E5:E13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Note: 'Italy' is a transit stamp (counted as Transit, not a visit). Schengen trip 15-27 Jul 2024 likely covered more countries than stamped - add them to the Travel Log from your itinerary.</t>
+      <c r="B18" s="4">
+        <f>SUM(B5:B16)</f>
+        <v/>
+      </c>
+      <c r="E18" s="4">
+        <f>SUM(E5:E16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Schengen trip 15-27 Jul 2024: France (entry CDG), Belgium, Netherlands, Switzerland, Italy/Rome (exit Milan) - internal borders are not stamped, so per-country dates are blank until you add them.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A20:F20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Germany to Jul 2024 Schengen trip
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MuHAkrVAM6ipkG9EkAQkug
</commit_message>
<xml_diff>
--- a/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
+++ b/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
@@ -19,7 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Method" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Travel Log'!$A$4:$L$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Travel Log'!$A$4:$L$84</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Access Map'!$A$4:$N$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Yatra Visa Planner'!$A$4:$K$36</definedName>
   </definedNames>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B14" s="6">
-        <f>COUNTIF('Country Summary'!B5:B16,"&gt;0")</f>
+        <f>COUNTIF('Country Summary'!B5:B17,"&gt;0")</f>
         <v/>
       </c>
       <c r="C14" t="inlineStr">
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="B15" s="6">
-        <f>'Country Summary'!B18</f>
+        <f>'Country Summary'!B19</f>
         <v/>
       </c>
       <c r="C15" t="inlineStr">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="B16" s="6">
-        <f>MAX('Country Summary'!B5:B16)</f>
+        <f>MAX('Country Summary'!B5:B17)</f>
         <v/>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -969,7 +969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="L16" s="9" t="inlineStr">
         <is>
-          <t>Schengen trip 15-27 Jul 2024 covering France, Belgium, Netherlands, Switzerland, Italy; France dates = whole-trip window, split per country when known</t>
+          <t>Schengen trip 15-27 Jul 2024 covering France, Belgium, Netherlands, Germany, Switzerland, Italy; France dates = whole-trip window, split per country when known</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C19" s="10" t="n"/>
@@ -1861,13 +1861,11 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n">
-        <v>45500</v>
-      </c>
+      <c r="D20" s="10" t="n"/>
       <c r="E20" s="9">
         <f>IF(AND(ISNUMBER(C20),ISNUMBER(D20)),D20-C20+1,"")</f>
         <v/>
@@ -1879,12 +1877,12 @@
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>By road/rail within Schengen (Rome visited)</t>
+          <t>By road/rail within Schengen (no stamp)</t>
         </is>
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>Milan Malpensa (MXP) -&gt; London Gatwick</t>
+          <t>By road/rail within Schengen (no stamp)</t>
         </is>
       </c>
       <c r="I20" s="9" t="inlineStr">
@@ -1894,7 +1892,7 @@
       </c>
       <c r="J20" s="9" t="inlineStr">
         <is>
-          <t>Your confirmation (Oct 2026): Rome visited; Passport p.17: Malpensa exit stamp 27 Jul 2024</t>
+          <t>Your confirmation (Oct 2026): visited during the 15-27 Jul 2024 Europe trip</t>
         </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
@@ -1904,7 +1902,7 @@
       </c>
       <c r="L20" s="9" t="inlineStr">
         <is>
-          <t>Entry date unknown - within 15-27 Jul 2024; departed Schengen from Milan</t>
+          <t>Dates unknown - within 15-27 Jul 2024; add from itinerary</t>
         </is>
       </c>
     </row>
@@ -1914,13 +1912,13 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="n">
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n">
         <v>45500</v>
       </c>
-      <c r="D21" s="10" t="n"/>
       <c r="E21" s="9">
         <f>IF(AND(ISNUMBER(C21),ISNUMBER(D21)),D21-C21+1,"")</f>
         <v/>
@@ -1932,32 +1930,32 @@
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>London Gatwick</t>
+          <t>By road/rail within Schengen (Rome visited)</t>
         </is>
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>(UK does not stamp exit)</t>
+          <t>Milan Malpensa (MXP) -&gt; London Gatwick</t>
         </is>
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>UK Standard Visitor C-visit, multiple, 29 Jun-29 Dec 2024</t>
+          <t>Schengen C visa #1</t>
         </is>
       </c>
       <c r="J21" s="9" t="inlineStr">
         <is>
-          <t>Passport p.23: Gatwick stamp 27 Jul 2024</t>
-        </is>
-      </c>
-      <c r="K21" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>Your confirmation (Oct 2026): Rome visited; Passport p.17: Malpensa exit stamp 27 Jul 2024</t>
+        </is>
+      </c>
+      <c r="K21" s="11" t="inlineStr">
+        <is>
+          <t>Check</t>
         </is>
       </c>
       <c r="L21" s="9" t="inlineStr">
         <is>
-          <t>Left UK by 01 Aug 2024 (UAE entry)</t>
+          <t>Entry date unknown - within 15-27 Jul 2024; departed Schengen from Milan</t>
         </is>
       </c>
     </row>
@@ -1967,11 +1965,11 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C22" s="12" t="n">
-        <v>45505</v>
+        <v>45500</v>
       </c>
       <c r="D22" s="10" t="n"/>
       <c r="E22" s="9">
@@ -1985,22 +1983,22 @@
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>Dubai Intl (DXB)</t>
+          <t>London Gatwick</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
-          <t>(UAE does not stamp exit)</t>
+          <t>(UK does not stamp exit)</t>
         </is>
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Visa/entry per stamp (Indian PP)</t>
+          <t>UK Standard Visitor C-visit, multiple, 29 Jun-29 Dec 2024</t>
         </is>
       </c>
       <c r="J22" s="9" t="inlineStr">
         <is>
-          <t>Passport p.10: UAE entry stamp 01 Aug 2024; India arrival RGI Hyderabad 05 Aug 2024</t>
+          <t>Passport p.23: Gatwick stamp 27 Jul 2024</t>
         </is>
       </c>
       <c r="K22" s="9" t="inlineStr">
@@ -2010,7 +2008,7 @@
       </c>
       <c r="L22" s="9" t="inlineStr">
         <is>
-          <t>Stayed up to ~4 days</t>
+          <t>Left UK by 01 Aug 2024 (UAE entry)</t>
         </is>
       </c>
     </row>
@@ -2020,15 +2018,13 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="C23" s="12" t="n">
-        <v>45904</v>
-      </c>
-      <c r="D23" s="12" t="n">
-        <v>45930</v>
-      </c>
+        <v>45505</v>
+      </c>
+      <c r="D23" s="10" t="n"/>
       <c r="E23" s="9">
         <f>IF(AND(ISNUMBER(C23),ISNUMBER(D23)),D23-C23+1,"")</f>
         <v/>
@@ -2040,39 +2036,94 @@
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
+          <t>Dubai Intl (DXB)</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>(UAE does not stamp exit)</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>Visa/entry per stamp (Indian PP)</t>
+        </is>
+      </c>
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>Passport p.10: UAE entry stamp 01 Aug 2024; India arrival RGI Hyderabad 05 Aug 2024</t>
+        </is>
+      </c>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="inlineStr">
+        <is>
+          <t>Stayed up to ~4 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="n">
+        <v>45904</v>
+      </c>
+      <c r="D24" s="12" t="n">
+        <v>45930</v>
+      </c>
+      <c r="E24" s="9">
+        <f>IF(AND(ISNUMBER(C24),ISNUMBER(D24)),D24-C24+1,"")</f>
+        <v/>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Visit</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
           <t>USA (CBP admitted 04 Sep 2025)</t>
         </is>
       </c>
-      <c r="H23" s="9" t="inlineStr">
+      <c r="H24" s="9" t="inlineStr">
         <is>
           <t>USA -&gt; Mumbai</t>
         </is>
       </c>
-      <c r="I23" s="9" t="inlineStr">
+      <c r="I24" s="9" t="inlineStr">
         <is>
           <t>B1/B2 10-yr visa (admitted until 03 Mar 2026)</t>
         </is>
       </c>
-      <c r="J23" s="9" t="inlineStr">
+      <c r="J24" s="9" t="inlineStr">
         <is>
           <t>Passport p.26 + p.10: India dep. New Delhi 03 Sep 2025; CBP stamp 04 Sep 2025; India arrival Mumbai 30 Sep 2025</t>
         </is>
       </c>
-      <c r="K23" s="9" t="inlineStr">
+      <c r="K24" s="9" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="L23" s="9" t="inlineStr">
+      <c r="L24" s="9" t="inlineStr">
         <is>
           <t>First use of US visa</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L83"/>
+  <autoFilter ref="A4:L84"/>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Visit,Transit"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2087,7 +2138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2151,19 +2202,19 @@
         </is>
       </c>
       <c r="B5" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A5,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A5,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A5,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A5,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A5,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A5,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A5,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A5,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A5,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A5,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E5" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A5,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A5,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="F5" s="9" t="inlineStr">
@@ -2179,19 +2230,19 @@
         </is>
       </c>
       <c r="B6" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A6,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A6,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A6,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A6,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A6,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A6,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A6,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A6,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A6,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A6,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A6,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A6,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -2207,19 +2258,19 @@
         </is>
       </c>
       <c r="B7" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A7,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A7,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A7,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A7,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A7,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A7,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A7,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A7,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A7,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A7,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E7" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A7,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A7,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="F7" s="9" t="inlineStr">
@@ -2231,23 +2282,23 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B8" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A8,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A8,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A8,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A8,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A8,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A8,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A8,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A8,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A8,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A8,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A8,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A8,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="F8" s="9" t="inlineStr">
@@ -2259,252 +2310,280 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Nepal</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B9" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A9,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A9,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A9,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A9,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A9,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A9,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A9,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A9,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A9,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A9,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E9" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A9,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A9,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>No visa needed; No visa needed (Indian PP)</t>
+          <t>Schengen C visa #1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Nepal</t>
         </is>
       </c>
       <c r="B10" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A10,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A10,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A10,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A10,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A10,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A10,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A10,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A10,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A10,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A10,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A10,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A10,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Schengen C visa #1</t>
+          <t>No visa needed; No visa needed (Indian PP)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Sri Lanka</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="B11" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A11,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A11,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A11,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A11,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A11,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A11,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A11,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A11,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A11,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A11,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E11" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A11,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A11,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>ETA 30-day, 1st visit (exp 16/01/2020); ETA 30-day, 1st visit (exp 23/02/2022); ETA 30-day, 1st visit (exp 28/10/2019)</t>
+          <t>Schengen C visa #1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Sri Lanka</t>
         </is>
       </c>
       <c r="B12" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A12,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A12,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="C12" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A12,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A12,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A12,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A12,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D12" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A12,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A12,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A12,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A12,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A12,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A12,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Schengen C visa #1</t>
+          <t>ETA 30-day, 1st visit (exp 16/01/2020); ETA 30-day, 1st visit (exp 23/02/2022); ETA 30-day, 1st visit (exp 28/10/2019)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="B13" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A13,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A13,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="C13" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A13,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A13,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A13,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A13,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D13" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A13,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A13,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A13,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A13,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E13" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A13,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A13,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>Visa on Arrival; Visa on Arrival (30 days)</t>
+          <t>Schengen C visa #1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="B14" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A14,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A14,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="C14" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A14,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A14,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A14,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A14,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D14" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A14,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A14,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A14,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A14,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A14,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A14,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Visa/entry per stamp (Indian PP)</t>
+          <t>Visa on Arrival; Visa on Arrival (30 days)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="B15" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A15,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A15,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="C15" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A15,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A15,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A15,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A15,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D15" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A15,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A15,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A15,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A15,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E15" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A15,'Travel Log'!$F$5:$F$83,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A15,'Travel Log'!$F$5:$F$84,"Visit")</f>
         <v/>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>B1/B2 10-yr visa (admitted until 03 Mar 2026)</t>
+          <t>Visa/entry per stamp (Indian PP)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="B16" s="9">
+        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A16,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <v/>
+      </c>
+      <c r="C16" s="12">
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A16,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A16,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="D16" s="12">
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A16,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A16,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="E16" s="9">
+        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A16,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <v/>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>B1/B2 10-yr visa (admitted until 03 Mar 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B16" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$83,A16,'Travel Log'!$F$5:$F$83,"Visit")</f>
-        <v/>
-      </c>
-      <c r="C16" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A16,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A16,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
-        <v/>
-      </c>
-      <c r="D16" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$83,A16,'Travel Log'!$C$5:$C$83,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$83,'Travel Log'!$B$5:$B$83,A16,'Travel Log'!$C$5:$C$83,"&gt;0"))</f>
-        <v/>
-      </c>
-      <c r="E16" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$83,'Travel Log'!$B$5:$B$83,A16,'Travel Log'!$F$5:$F$83,"Visit")</f>
-        <v/>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="B17" s="9">
+        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A17,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <v/>
+      </c>
+      <c r="C17" s="12">
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A17,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A17,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="D17" s="12">
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A17,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A17,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="E17" s="9">
+        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A17,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <v/>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>UK Standard Visitor C-visit, multiple, 29 Jun-29 Dec 2024</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B18" s="4">
-        <f>SUM(B5:B16)</f>
-        <v/>
-      </c>
-      <c r="E18" s="4">
-        <f>SUM(E5:E16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>Schengen trip 15-27 Jul 2024: France (entry CDG), Belgium, Netherlands, Switzerland, Italy/Rome (exit Milan) - internal borders are not stamped, so per-country dates are blank until you add them.</t>
+      <c r="B19" s="4">
+        <f>SUM(B5:B17)</f>
+        <v/>
+      </c>
+      <c r="E19" s="4">
+        <f>SUM(E5:E17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Schengen trip 15-27 Jul 2024: France (entry CDG), Belgium, Netherlands, Germany, Switzerland, Italy/Rome (exit Milan) - internal borders are not stamped, so per-country dates are blank until you add them.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Vatican City to Jul 2024 Schengen trip
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MuHAkrVAM6ipkG9EkAQkug
</commit_message>
<xml_diff>
--- a/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
+++ b/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
@@ -19,7 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Method" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Travel Log'!$A$4:$L$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Travel Log'!$A$4:$L$85</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Access Map'!$A$4:$N$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Yatra Visa Planner'!$A$4:$K$36</definedName>
   </definedNames>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B14" s="6">
-        <f>COUNTIF('Country Summary'!B5:B17,"&gt;0")</f>
+        <f>COUNTIF('Country Summary'!B5:B18,"&gt;0")</f>
         <v/>
       </c>
       <c r="C14" t="inlineStr">
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="B15" s="6">
-        <f>'Country Summary'!B19</f>
+        <f>'Country Summary'!B20</f>
         <v/>
       </c>
       <c r="C15" t="inlineStr">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="B16" s="6">
-        <f>MAX('Country Summary'!B5:B17)</f>
+        <f>MAX('Country Summary'!B5:B18)</f>
         <v/>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -969,7 +969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="L16" s="9" t="inlineStr">
         <is>
-          <t>Schengen trip 15-27 Jul 2024 covering France, Belgium, Netherlands, Germany, Switzerland, Italy; France dates = whole-trip window, split per country when known</t>
+          <t>Schengen trip 15-27 Jul 2024 covering France, Belgium, Netherlands, Germany, Switzerland, Italy/Rome, Vatican City; France dates = whole-trip window, split per country when known</t>
         </is>
       </c>
     </row>
@@ -1912,13 +1912,11 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Vatican City</t>
         </is>
       </c>
       <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n">
-        <v>45500</v>
-      </c>
+      <c r="D21" s="10" t="n"/>
       <c r="E21" s="9">
         <f>IF(AND(ISNUMBER(C21),ISNUMBER(D21)),D21-C21+1,"")</f>
         <v/>
@@ -1930,22 +1928,22 @@
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>By road/rail within Schengen (Rome visited)</t>
+          <t>On foot from Rome (no border control)</t>
         </is>
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>Milan Malpensa (MXP) -&gt; London Gatwick</t>
+          <t>On foot from Rome (no border control)</t>
         </is>
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Schengen C visa #1</t>
+          <t>Schengen C visa #1 (Vatican has open border with Italy)</t>
         </is>
       </c>
       <c r="J21" s="9" t="inlineStr">
         <is>
-          <t>Your confirmation (Oct 2026): Rome visited; Passport p.17: Malpensa exit stamp 27 Jul 2024</t>
+          <t>Your confirmation (Oct 2026): visited from Rome during the 15-27 Jul 2024 Europe trip</t>
         </is>
       </c>
       <c r="K21" s="11" t="inlineStr">
@@ -1955,7 +1953,7 @@
       </c>
       <c r="L21" s="9" t="inlineStr">
         <is>
-          <t>Entry date unknown - within 15-27 Jul 2024; departed Schengen from Milan</t>
+          <t>Sovereign state; same day(s) as Rome - add date from itinerary</t>
         </is>
       </c>
     </row>
@@ -1965,13 +1963,13 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="C22" s="12" t="n">
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n">
         <v>45500</v>
       </c>
-      <c r="D22" s="10" t="n"/>
       <c r="E22" s="9">
         <f>IF(AND(ISNUMBER(C22),ISNUMBER(D22)),D22-C22+1,"")</f>
         <v/>
@@ -1983,32 +1981,32 @@
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>London Gatwick</t>
+          <t>By road/rail within Schengen (Rome visited)</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
-          <t>(UK does not stamp exit)</t>
+          <t>Milan Malpensa (MXP) -&gt; London Gatwick</t>
         </is>
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>UK Standard Visitor C-visit, multiple, 29 Jun-29 Dec 2024</t>
+          <t>Schengen C visa #1</t>
         </is>
       </c>
       <c r="J22" s="9" t="inlineStr">
         <is>
-          <t>Passport p.23: Gatwick stamp 27 Jul 2024</t>
-        </is>
-      </c>
-      <c r="K22" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>Your confirmation (Oct 2026): Rome visited; Passport p.17: Malpensa exit stamp 27 Jul 2024</t>
+        </is>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
+        <is>
+          <t>Check</t>
         </is>
       </c>
       <c r="L22" s="9" t="inlineStr">
         <is>
-          <t>Left UK by 01 Aug 2024 (UAE entry)</t>
+          <t>Entry date unknown - within 15-27 Jul 2024; departed Schengen from Milan</t>
         </is>
       </c>
     </row>
@@ -2018,11 +2016,11 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C23" s="12" t="n">
-        <v>45505</v>
+        <v>45500</v>
       </c>
       <c r="D23" s="10" t="n"/>
       <c r="E23" s="9">
@@ -2036,22 +2034,22 @@
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>Dubai Intl (DXB)</t>
+          <t>London Gatwick</t>
         </is>
       </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
-          <t>(UAE does not stamp exit)</t>
+          <t>(UK does not stamp exit)</t>
         </is>
       </c>
       <c r="I23" s="9" t="inlineStr">
         <is>
-          <t>Visa/entry per stamp (Indian PP)</t>
+          <t>UK Standard Visitor C-visit, multiple, 29 Jun-29 Dec 2024</t>
         </is>
       </c>
       <c r="J23" s="9" t="inlineStr">
         <is>
-          <t>Passport p.10: UAE entry stamp 01 Aug 2024; India arrival RGI Hyderabad 05 Aug 2024</t>
+          <t>Passport p.23: Gatwick stamp 27 Jul 2024</t>
         </is>
       </c>
       <c r="K23" s="9" t="inlineStr">
@@ -2061,7 +2059,7 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Stayed up to ~4 days</t>
+          <t>Left UK by 01 Aug 2024 (UAE entry)</t>
         </is>
       </c>
     </row>
@@ -2071,15 +2069,13 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="C24" s="12" t="n">
-        <v>45904</v>
-      </c>
-      <c r="D24" s="12" t="n">
-        <v>45930</v>
-      </c>
+        <v>45505</v>
+      </c>
+      <c r="D24" s="10" t="n"/>
       <c r="E24" s="9">
         <f>IF(AND(ISNUMBER(C24),ISNUMBER(D24)),D24-C24+1,"")</f>
         <v/>
@@ -2091,39 +2087,94 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
+          <t>Dubai Intl (DXB)</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>(UAE does not stamp exit)</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>Visa/entry per stamp (Indian PP)</t>
+        </is>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>Passport p.10: UAE entry stamp 01 Aug 2024; India arrival RGI Hyderabad 05 Aug 2024</t>
+        </is>
+      </c>
+      <c r="K24" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L24" s="9" t="inlineStr">
+        <is>
+          <t>Stayed up to ~4 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>45904</v>
+      </c>
+      <c r="D25" s="12" t="n">
+        <v>45930</v>
+      </c>
+      <c r="E25" s="9">
+        <f>IF(AND(ISNUMBER(C25),ISNUMBER(D25)),D25-C25+1,"")</f>
+        <v/>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>Visit</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
           <t>USA (CBP admitted 04 Sep 2025)</t>
         </is>
       </c>
-      <c r="H24" s="9" t="inlineStr">
+      <c r="H25" s="9" t="inlineStr">
         <is>
           <t>USA -&gt; Mumbai</t>
         </is>
       </c>
-      <c r="I24" s="9" t="inlineStr">
+      <c r="I25" s="9" t="inlineStr">
         <is>
           <t>B1/B2 10-yr visa (admitted until 03 Mar 2026)</t>
         </is>
       </c>
-      <c r="J24" s="9" t="inlineStr">
+      <c r="J25" s="9" t="inlineStr">
         <is>
           <t>Passport p.26 + p.10: India dep. New Delhi 03 Sep 2025; CBP stamp 04 Sep 2025; India arrival Mumbai 30 Sep 2025</t>
         </is>
       </c>
-      <c r="K24" s="9" t="inlineStr">
+      <c r="K25" s="9" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="L24" s="9" t="inlineStr">
+      <c r="L25" s="9" t="inlineStr">
         <is>
           <t>First use of US visa</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L84"/>
+  <autoFilter ref="A4:L85"/>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Visit,Transit"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2138,7 +2189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2202,19 +2253,19 @@
         </is>
       </c>
       <c r="B5" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A5,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$85,A5,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A5,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A5,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A5,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A5,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A5,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A5,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A5,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A5,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E5" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A5,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$85,'Travel Log'!$B$5:$B$85,A5,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="F5" s="9" t="inlineStr">
@@ -2230,19 +2281,19 @@
         </is>
       </c>
       <c r="B6" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A6,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$85,A6,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A6,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A6,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A6,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A6,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A6,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A6,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A6,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A6,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A6,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$85,'Travel Log'!$B$5:$B$85,A6,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -2258,19 +2309,19 @@
         </is>
       </c>
       <c r="B7" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A7,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$85,A7,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A7,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A7,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A7,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A7,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A7,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A7,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A7,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A7,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E7" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A7,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$85,'Travel Log'!$B$5:$B$85,A7,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="F7" s="9" t="inlineStr">
@@ -2286,19 +2337,19 @@
         </is>
       </c>
       <c r="B8" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A8,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$85,A8,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A8,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A8,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A8,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A8,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A8,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A8,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A8,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A8,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A8,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$85,'Travel Log'!$B$5:$B$85,A8,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="F8" s="9" t="inlineStr">
@@ -2314,19 +2365,19 @@
         </is>
       </c>
       <c r="B9" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A9,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$85,A9,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A9,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A9,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A9,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A9,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A9,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A9,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A9,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A9,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E9" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A9,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$85,'Travel Log'!$B$5:$B$85,A9,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="F9" s="9" t="inlineStr">
@@ -2342,19 +2393,19 @@
         </is>
       </c>
       <c r="B10" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A10,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$85,A10,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A10,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A10,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A10,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A10,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A10,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A10,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A10,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A10,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A10,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$85,'Travel Log'!$B$5:$B$85,A10,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="F10" s="9" t="inlineStr">
@@ -2370,19 +2421,19 @@
         </is>
       </c>
       <c r="B11" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A11,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$85,A11,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A11,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A11,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A11,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A11,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A11,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A11,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A11,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A11,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E11" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A11,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$85,'Travel Log'!$B$5:$B$85,A11,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="F11" s="9" t="inlineStr">
@@ -2398,19 +2449,19 @@
         </is>
       </c>
       <c r="B12" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A12,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$85,A12,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="C12" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A12,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A12,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A12,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A12,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D12" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A12,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A12,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A12,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A12,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A12,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$85,'Travel Log'!$B$5:$B$85,A12,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="F12" s="9" t="inlineStr">
@@ -2426,19 +2477,19 @@
         </is>
       </c>
       <c r="B13" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A13,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$85,A13,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="C13" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A13,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A13,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A13,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A13,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D13" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A13,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A13,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A13,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A13,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E13" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A13,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$85,'Travel Log'!$B$5:$B$85,A13,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="F13" s="9" t="inlineStr">
@@ -2454,19 +2505,19 @@
         </is>
       </c>
       <c r="B14" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A14,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$85,A14,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="C14" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A14,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A14,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A14,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A14,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D14" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A14,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A14,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A14,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A14,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A14,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$85,'Travel Log'!$B$5:$B$85,A14,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -2482,19 +2533,19 @@
         </is>
       </c>
       <c r="B15" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A15,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$85,A15,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="C15" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A15,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A15,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A15,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A15,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D15" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A15,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A15,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A15,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A15,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E15" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A15,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$85,'Travel Log'!$B$5:$B$85,A15,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -2510,19 +2561,19 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A16,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$85,A16,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="C16" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A16,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A16,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A16,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A16,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A16,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A16,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A16,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A16,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E16" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A16,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$85,'Travel Log'!$B$5:$B$85,A16,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="F16" s="9" t="inlineStr">
@@ -2538,19 +2589,19 @@
         </is>
       </c>
       <c r="B17" s="9">
-        <f>COUNTIFS('Travel Log'!$B$5:$B$84,A17,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>COUNTIFS('Travel Log'!$B$5:$B$85,A17,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="C17" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A17,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A17,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A17,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A17,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$84,A17,'Travel Log'!$C$5:$C$84,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$84,'Travel Log'!$B$5:$B$84,A17,'Travel Log'!$C$5:$C$84,"&gt;0"))</f>
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A17,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A17,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E17" s="9">
-        <f>SUMIFS('Travel Log'!$E$5:$E$84,'Travel Log'!$B$5:$B$84,A17,'Travel Log'!$F$5:$F$84,"Visit")</f>
+        <f>SUMIFS('Travel Log'!$E$5:$E$85,'Travel Log'!$B$5:$B$85,A17,'Travel Log'!$F$5:$F$85,"Visit")</f>
         <v/>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -2559,31 +2610,59 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Vatican City</t>
+        </is>
+      </c>
+      <c r="B18" s="9">
+        <f>COUNTIFS('Travel Log'!$B$5:$B$85,A18,'Travel Log'!$F$5:$F$85,"Visit")</f>
+        <v/>
+      </c>
+      <c r="C18" s="12">
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A18,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MINIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A18,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="D18" s="12">
+        <f>IF(COUNTIFS('Travel Log'!$B$5:$B$85,A18,'Travel Log'!$C$5:$C$85,"&gt;0")=0,"",_xlfn.MAXIFS('Travel Log'!$C$5:$C$85,'Travel Log'!$B$5:$B$85,A18,'Travel Log'!$C$5:$C$85,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="E18" s="9">
+        <f>SUMIFS('Travel Log'!$E$5:$E$85,'Travel Log'!$B$5:$B$85,A18,'Travel Log'!$F$5:$F$85,"Visit")</f>
+        <v/>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Schengen C visa #1 (Vatican has open border with Italy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B19" s="4">
-        <f>SUM(B5:B17)</f>
-        <v/>
-      </c>
-      <c r="E19" s="4">
-        <f>SUM(E5:E17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="45" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>Schengen trip 15-27 Jul 2024: France (entry CDG), Belgium, Netherlands, Germany, Switzerland, Italy/Rome (exit Milan) - internal borders are not stamped, so per-country dates are blank until you add them.</t>
+      <c r="B20" s="4">
+        <f>SUM(B5:B18)</f>
+        <v/>
+      </c>
+      <c r="E20" s="4">
+        <f>SUM(E5:E18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Schengen trip 15-27 Jul 2024: France (entry CDG), Belgium, Netherlands, Germany, Switzerland, Italy/Rome + Vatican City (exit Milan) - internal borders are not stamped, so per-country dates are blank until you add them.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A22:F22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Yatra Wishlist section (Mysore Dasara, Tirupati Brahmotsavam, Vaishno Devi, Amarnath, Seven Sisters, Kerala)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MuHAkrVAM6ipkG9EkAQkug
</commit_message>
<xml_diff>
--- a/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
+++ b/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
@@ -14,14 +14,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access Map" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power Visas" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatra Visa Planner" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="To Confirm" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alerts" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Method" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatra Wishlist" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="To Confirm" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alerts" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Method" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Travel Log'!$A$4:$L$85</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Access Map'!$A$4:$N$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Yatra Visa Planner'!$A$4:$K$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Yatra Wishlist'!$A$4:$N$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -561,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -791,93 +793,109 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Valid visas right now</t>
+          <t>Wishlist ideas (open)</t>
         </is>
       </c>
       <c r="B18" s="6">
-        <f>COUNTIF('Visas Held'!H5:H30,"VALID")</f>
-        <v/>
-      </c>
-      <c r="C18" t="inlineStr"/>
+        <f>COUNTIFS('Yatra Wishlist'!K5:K200,"&lt;&gt;Done",'Yatra Wishlist'!K5:K200,"&lt;&gt;Dropped",'Yatra Wishlist'!B5:B200,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>See Yatra Wishlist</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>Valid visas right now</t>
+        </is>
+      </c>
+      <c r="B19" s="6">
+        <f>COUNTIF('Visas Held'!H5:H30,"VALID")</f>
+        <v/>
+      </c>
+      <c r="C19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>Expired visas to renew</t>
         </is>
       </c>
-      <c r="B19" s="6">
+      <c r="B20" s="6">
         <f>COUNTIF('Visas Held'!H5:H30,"EXPIRED")</f>
         <v/>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Schengen &amp; UK</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>Top actions</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="48" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>Passport expires 17 Sep 2028</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Most countries need 6 months validity -&gt; practical last safe travel date ~17 Mar 2028. Start renewal ~Sep 2027. Passports issued in India are e-passports since 28 May 2025. Keep old passport: US &amp; Australia visas stay valid but must be carried; tell Australia Home Affairs new passport number (ImmiAccount).</t>
         </is>
       </c>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Schengen: no valid visa</t>
+          <t>Passport expires 17 Sep 2028</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Both France visas expired (Apr 2026). You now have 2 lawful visas in 3 years -&gt; eligible for the EU 'cascade' 2-year multiple-entry visa. Apply 3 months before the next Europe yatra.</t>
+          <t>Most countries need 6 months validity -&gt; practical last safe travel date ~17 Mar 2028. Start renewal ~Sep 2027. Passports issued in India are e-passports since 28 May 2025. Keep old passport: US &amp; Australia visas stay valid but must be carried; tell Australia Home Affairs new passport number (ImmiAccount).</t>
         </is>
       </c>
     </row>
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>UK: no valid visa</t>
+          <t>Schengen: no valid visa</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>UK visa expired 29 Dec 2024. Apply 3-4 weeks ahead; consider a 2-year or 5-year Standard Visitor visa if you will return often.</t>
+          <t>Both France visas expired (Apr 2026). You now have 2 lawful visas in 3 years -&gt; eligible for the EU 'cascade' 2-year multiple-entry visa. Apply 3 months before the next Europe yatra.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Australia: confirm stream</t>
+          <t>UK: no valid visa</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Visa is Business Visitor stream (condition 8115). A pilgrimage yatra with devotees may count as tourism - confirm whether to apply for a Tourist-stream visa.</t>
+          <t>UK visa expired 29 Dec 2024. Apply 3-4 weeks ahead; consider a 2-year or 5-year Standard Visitor visa if you will return often.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
         <is>
+          <t>Australia: confirm stream</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Visa is Business Visitor stream (condition 8115). A pilgrimage yatra with devotees may count as tourism - confirm whether to apply for a Tourist-stream visa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
           <t>Malaysia visa-free ends 31 Dec 2026</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>Get visa/e-visa for any 2027 Malaysia yatra unless extended.</t>
         </is>
@@ -889,6 +907,202 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001F2A44"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Alerts &amp; action items</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Review every month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Alert</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Passport expires 17 Sep 2028</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Most countries need 6 months validity -&gt; practical last safe travel date ~17 Mar 2028. Start renewal ~Sep 2027. Passports issued in India are e-passports since 28 May 2025. Keep old passport: US &amp; Australia visas stay valid but must be carried; tell Australia Home Affairs new passport number (ImmiAccount).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Schengen: no valid visa</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Both France visas expired (Apr 2026). You now have 2 lawful visas in 3 years -&gt; eligible for the EU 'cascade' 2-year multiple-entry visa. Apply 3 months before the next Europe yatra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>UK: no valid visa</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>UK visa expired 29 Dec 2024. Apply 3-4 weeks ahead; consider a 2-year or 5-year Standard Visitor visa if you will return often.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Australia: confirm stream</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Visa is Business Visitor stream (condition 8115). A pilgrimage yatra with devotees may count as tourism - confirm whether to apply for a Tourist-stream visa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Malaysia visa-free ends 31 Dec 2026</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Get visa/e-visa for any 2027 Malaysia yatra unless extended.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Thailand now 30 days (from 15 Sep 2026, reported)</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Plan group stays accordingly; complete TDAC before arrival.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Mismatches found between your sheets and the documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Schengen #1 duration</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Your 'Visa' tab says 45 days; the visa sticker says 30 days (valid 15-Jul-24 to 29-Aug-24).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Schengen #2 duration</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Sticker: 30 days within 21-Oct-25 to 19-Apr-26 (your tab shows 180 = validity window, not stay).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>US visa stay</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Your tab shows 3,647 days = visa validity. Stay per entry is set by CBP at the port (I-94), not by the visa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Your tab says 'Business'. VEVO confirms Business Visitor stream (conditions 8115/8201). Tourism/pilgrimage may need Tourist stream.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Old access lists</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Armenia 'UK visa 120 days', Bosnia '30 days', Montenegro 'US 15 days', Turkey/Qatar/Kuwait entries were out of date - corrected in Access Map.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Hong Kong / Barbados etc.</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Your 'Indian PP visa on arrival' rows were not re-researched except those listed in the Yatra Visa Planner. Treat as unverified.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001F2A44"/>
@@ -7644,6 +7858,506 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Yatra Wishlist - places to visit, explore and plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Live list: add a row per idea; set Status from the dropdown. Dates/permits are planning notes - confirm each year's official calendar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Yatra / place</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Best time</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Typical dates / festival window</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Visa / permit / registration</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Notes &amp; highlights</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Target year</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Next step</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Added on</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Mysore Dasara</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Mysuru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Festival yatra</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Sep-Oct (Navaratri)</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>10 days ending Vijayadashami; Jamboo Savari on the last day</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>None (domestic)</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>Palace illumination, Chamundi Hill, Jamboo Savari procession. Book stay months ahead; ISKCON Mysore nearby. Combine with Srirangapatna, Melukote.</t>
+        </is>
+      </c>
+      <c r="J5" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K5" s="19" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="L5" s="19" t="inlineStr"/>
+      <c r="M5" s="19" t="inlineStr"/>
+      <c r="N5" s="12" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Tirupati Balaji Brahmotsavam</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Tirumala, Andhra Pradesh, India</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Festival yatra</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Sep-Oct (Salakatla Brahmotsavam); some years a 2nd Navaratri Brahmotsavam</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>9 days; Garuda Seva day is the peak</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>None; TTD darshan tokens / SED booking via tirupatibalaji.ap.gov.in</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>Vahana sevas each morning/evening; Garuda Seva night draws lakhs. Arrange accommodation via TTD or HKM contacts well in advance.</t>
+        </is>
+      </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K6" s="19" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="L6" s="19" t="inlineStr"/>
+      <c r="M6" s="19" t="inlineStr"/>
+      <c r="N6" s="12" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Vaishno Devi</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Katra, Jammu &amp; Kashmir, India</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Shakti-peetha trek</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Mar-Jun and Sep-Nov (avoid peak summer rush and Jan snow)</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Navaratri very crowded</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>3-4 (with travel)</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>None; free RFID yatra card from SMVDSB (online or Katra)</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>13 km trek from Katra (ponies/palki/helicopter available). Combine with Jammu Raghunath temple; optionally Amritsar.</t>
+        </is>
+      </c>
+      <c r="J7" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K7" s="19" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="L7" s="19" t="inlineStr"/>
+      <c r="M7" s="19" t="inlineStr"/>
+      <c r="N7" s="12" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Amarnath Yatra</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Pahalgam / Baltal, Jammu &amp; Kashmir, India</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>High-altitude cave pilgrimage</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Jul-Aug only (yatra window set yearly by SASB)</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>~45-60 days, Ashadha Purnima to Shravana Purnima (Raksha Bandhan)</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Compulsory SASB registration + Compulsory Health Certificate from authorised doctor; RFID card; age 13-70</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Register as soon as the window opens (Mar-Apr). Pahalgam route 32 km (3 days) or Baltal 14 km (1 day); helicopter options. Needs fitness prep.</t>
+        </is>
+      </c>
+      <c r="J8" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K8" s="19" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="L8" s="19" t="inlineStr"/>
+      <c r="M8" s="19" t="inlineStr"/>
+      <c r="N8" s="12" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Seven Sisters (North-East India)</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Assam, Meghalaya, Arunachal, Nagaland, Manipur, Mizoram, Tripura</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Multi-state exploration yatra</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Oct-Apr (dry, clear)</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Avoid Jun-Sep monsoon</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>10-14</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>Inner Line Permit (ILP) for Arunachal, Nagaland, Mizoram, Manipur - online; none for Assam/Meghalaya/Tripura</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>Kamakhya (Guwahati), Majuli satras (Vaishnava), Tawang monastery, Cherrapunji/Living root bridges, Loktak lake, Tripureshwari temple. Plan as 2 circuits (Assam-Meghalaya-Arunachal; Manipur-Mizoram-Tripura-Nagaland).</t>
+        </is>
+      </c>
+      <c r="J9" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K9" s="19" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="L9" s="19" t="inlineStr"/>
+      <c r="M9" s="19" t="inlineStr"/>
+      <c r="N9" s="12" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Kerala</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Kerala, India</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Temple + culture yatra</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Oct-Mar; Sabarimala season Nov-Jan</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Guruvayur Ekadasi (Nov-Dec); Thrissur Pooram (Apr-May)</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>None (domestic); Sabarimala needs virtual-queue booking</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>Guruvayur, Padmanabhaswamy (dress code), Sabarimala, Ambalappuzha, Aranmula, Chottanikkara; backwaters. Combine with Kanyakumari/Suchindram.</t>
+        </is>
+      </c>
+      <c r="J10" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K10" s="19" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="L10" s="19" t="inlineStr"/>
+      <c r="M10" s="19" t="inlineStr"/>
+      <c r="N10" s="12" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:N110"/>
+  <conditionalFormatting sqref="K5:K110">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
+      <formula>"Done"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="2">
+      <formula>"Booked"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
+      <formula>"Planned"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="0">
+      <formula>"Dropped"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="K5:K110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Idea,Researching,Planned,Booked,Done,Dropped"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J5:J110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"High,Medium,Low"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001F2A44"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8000,200 +8714,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="001F2A44"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Alerts &amp; action items</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Review every month.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Alert</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>What to do</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Passport expires 17 Sep 2028</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Most countries need 6 months validity -&gt; practical last safe travel date ~17 Mar 2028. Start renewal ~Sep 2027. Passports issued in India are e-passports since 28 May 2025. Keep old passport: US &amp; Australia visas stay valid but must be carried; tell Australia Home Affairs new passport number (ImmiAccount).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Schengen: no valid visa</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Both France visas expired (Apr 2026). You now have 2 lawful visas in 3 years -&gt; eligible for the EU 'cascade' 2-year multiple-entry visa. Apply 3 months before the next Europe yatra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>UK: no valid visa</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>UK visa expired 29 Dec 2024. Apply 3-4 weeks ahead; consider a 2-year or 5-year Standard Visitor visa if you will return often.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>Australia: confirm stream</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>Visa is Business Visitor stream (condition 8115). A pilgrimage yatra with devotees may count as tourism - confirm whether to apply for a Tourist-stream visa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>Malaysia visa-free ends 31 Dec 2026</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Get visa/e-visa for any 2027 Malaysia yatra unless extended.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>Thailand now 30 days (from 15 Sep 2026, reported)</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Plan group stays accordingly; complete TDAC before arrival.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="17" t="inlineStr">
-        <is>
-          <t>Mismatches found between your sheets and the documents</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Schengen #1 duration</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Your 'Visa' tab says 45 days; the visa sticker says 30 days (valid 15-Jul-24 to 29-Aug-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>Schengen #2 duration</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Sticker: 30 days within 21-Oct-25 to 19-Apr-26 (your tab shows 180 = validity window, not stay).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>US visa stay</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Your tab shows 3,647 days = visa validity. Stay per entry is set by CBP at the port (I-94), not by the visa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Your tab says 'Business'. VEVO confirms Business Visitor stream (conditions 8115/8201). Tourism/pilgrimage may need Tourist stream.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>Old access lists</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Armenia 'UK visa 120 days', Bosnia '30 days', Montenegro 'US 15 days', Turkey/Qatar/Kuwait entries were out of date - corrected in Access Map.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>Hong Kong / Barbados etc.</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Your 'Indian PP visa on arrival' rows were not re-researched except those listed in the Yatra Visa Planner. Treat as unverified.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Pune and Indore/Madhya Pradesh to Yatra Wishlist
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MuHAkrVAM6ipkG9EkAQkug
</commit_message>
<xml_diff>
--- a/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
+++ b/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Travel Log'!$A$4:$L$85</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Access Map'!$A$4:$N$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Yatra Visa Planner'!$A$4:$K$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Yatra Wishlist'!$A$4:$N$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Yatra Wishlist'!$A$4:$N$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -7858,7 +7858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8269,42 +8269,42 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Kerala</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Kerala, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Temple + culture yatra</t>
+          <t>City + temple exploration</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Oct-Mar; Sabarimala season Nov-Jan</t>
+          <t>Oct-Feb (pleasant); Ganesh Chaturthi (Aug-Sep) for the festival</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Guruvayur Ekadasi (Nov-Dec); Thrissur Pooram (Apr-May)</t>
+          <t>Ganeshotsav 10 days ending Anant Chaturdashi</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>6-8</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>None (domestic); Sabarimala needs virtual-queue booking</t>
+          <t>None (domestic)</t>
         </is>
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>Guruvayur, Padmanabhaswamy (dress code), Sabarimala, Ambalappuzha, Aranmula, Chottanikkara; backwaters. Combine with Kanyakumari/Suchindram.</t>
+          <t>ISKCON NVCC (Katraj) and ISKCON Camp; Dagdusheth Halwai Ganapati; Alandi (Dnyaneshwar samadhi) and Dehu (Tukaram) - Warkari heritage; Jejuri Khandoba; Bhimashankar Jyotirlinga day trip; Shaniwar Wada, Parvati hill. Can combine with Pandharpur (Ashadhi Ekadashi) or Shirdi.</t>
         </is>
       </c>
       <c r="J10" s="19" t="inlineStr">
@@ -8323,9 +8323,129 @@
         <v>46316</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Indore &amp; Madhya Pradesh</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Indore / Ujjain / Omkareshwar / Maheshwar, Madhya Pradesh, India</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Jyotirlinga + heritage yatra</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Oct-Mar (avoid Apr-Jun heat)</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Ujjain Simhastha Kumbh next due 2028 (Apr-May); Mahakal Bhasma Aarti daily at ~4 am (book online)</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>None (domestic); Bhasma Aarti permission via shrimahakaleshwar.com</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>Base at Indore (Khajrana Ganesh, ISKCON Indore, Sarafa night food street). Ujjain: Mahakaleshwar + Mahakal Lok corridor, Kal Bhairav, Sandipani Ashram (Krishna's school). Omkareshwar Jyotirlinga + parikrama; Maheshwar ghats (Ahilyabai); Mandu. Optional extension: Chitrakoot / Khajuraho / Sanchi. Plan a 2028 Simhastha batch separately.</t>
+        </is>
+      </c>
+      <c r="J11" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K11" s="19" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="L11" s="19" t="inlineStr"/>
+      <c r="M11" s="19" t="inlineStr"/>
+      <c r="N11" s="12" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Kerala</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Kerala, India</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Temple + culture yatra</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Oct-Mar; Sabarimala season Nov-Jan</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Guruvayur Ekadasi (Nov-Dec); Thrissur Pooram (Apr-May)</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>None (domestic); Sabarimala needs virtual-queue booking</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Guruvayur, Padmanabhaswamy (dress code), Sabarimala, Ambalappuzha, Aranmula, Chottanikkara; backwaters. Combine with Kanyakumari/Suchindram.</t>
+        </is>
+      </c>
+      <c r="J12" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K12" s="19" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="L12" s="19" t="inlineStr"/>
+      <c r="M12" s="19" t="inlineStr"/>
+      <c r="N12" s="12" t="n">
+        <v>46316</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:N110"/>
-  <conditionalFormatting sqref="K5:K110">
+  <autoFilter ref="A4:N112"/>
+  <conditionalFormatting sqref="K5:K112">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>"Done"</formula>
     </cfRule>
@@ -8340,10 +8460,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="K5:K110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K5:K112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Idea,Researching,Planned,Booked,Done,Dropped"</formula1>
     </dataValidation>
-    <dataValidation sqref="J5:J110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J5:J112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add Mumbai NMACC to Yatra Wishlist
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MuHAkrVAM6ipkG9EkAQkug
</commit_message>
<xml_diff>
--- a/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
+++ b/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Travel Log'!$A$4:$L$85</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Access Map'!$A$4:$N$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Yatra Visa Planner'!$A$4:$K$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Yatra Wishlist'!$A$4:$N$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Yatra Wishlist'!$A$4:$N$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -7858,7 +7858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8389,42 +8389,42 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Kerala</t>
+          <t>Mumbai - NMACC (Nita Mukesh Ambani Cultural Centre)</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Kerala, India</t>
+          <t>BKC, Mumbai, Maharashtra, India</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Temple + culture yatra</t>
+          <t>Culture + temple exploration</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>Oct-Mar; Sabarimala season Nov-Jan</t>
+          <t>Oct-Feb (dry season); check NMACC programme calendar for shows/exhibitions</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Guruvayur Ekadasi (Nov-Dec); Thrissur Pooram (Apr-May)</t>
+          <t>Year-round; 'Swadesh' crafts exhibition is permanent, theatre shows are ticketed</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>6-8</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>None (domestic); Sabarimala needs virtual-queue booking</t>
+          <t>None (domestic); NMACC show tickets via nmacc.com / BookMyShow</t>
         </is>
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>Guruvayur, Padmanabhaswamy (dress code), Sabarimala, Ambalappuzha, Aranmula, Chottanikkara; backwaters. Combine with Kanyakumari/Suchindram.</t>
+          <t>NMACC: Grand Theatre, Studio Theatre, Cube, Art House exhibitions, Swadesh artisan showcase. Combine with ISKCON Juhu (Prabhupada samadhi/museum), ISKCON Chowpatty (Radha Gopinath), Siddhivinayak, Mahalakshmi, Babulnath, Mumba Devi; Elephanta caves day trip. Was already on your Bucket List tab.</t>
         </is>
       </c>
       <c r="J12" s="19" t="inlineStr">
@@ -8443,9 +8443,69 @@
         <v>46316</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Kerala</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Kerala, India</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Temple + culture yatra</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Oct-Mar; Sabarimala season Nov-Jan</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Guruvayur Ekadasi (Nov-Dec); Thrissur Pooram (Apr-May)</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>None (domestic); Sabarimala needs virtual-queue booking</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>Guruvayur, Padmanabhaswamy (dress code), Sabarimala, Ambalappuzha, Aranmula, Chottanikkara; backwaters. Combine with Kanyakumari/Suchindram.</t>
+        </is>
+      </c>
+      <c r="J13" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K13" s="19" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="L13" s="19" t="inlineStr"/>
+      <c r="M13" s="19" t="inlineStr"/>
+      <c r="N13" s="12" t="n">
+        <v>46316</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:N112"/>
-  <conditionalFormatting sqref="K5:K112">
+  <autoFilter ref="A4:N113"/>
+  <conditionalFormatting sqref="K5:K113">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>"Done"</formula>
     </cfRule>
@@ -8460,10 +8520,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="K5:K112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K5:K113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Idea,Researching,Planned,Booked,Done,Dropped"</formula1>
     </dataValidation>
-    <dataValidation sqref="J5:J112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J5:J113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add Places Visited master list from Europe+London itinerary; infer per-country dates for Jul 2024 trip
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MuHAkrVAM6ipkG9EkAQkug
</commit_message>
<xml_diff>
--- a/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
+++ b/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
@@ -14,16 +14,18 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access Map" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power Visas" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatra Visa Planner" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatra Wishlist" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="To Confirm" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alerts" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Method" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Places Visited" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatra Wishlist" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="To Confirm" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alerts" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Method" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Travel Log'!$A$4:$L$85</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Access Map'!$A$4:$N$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Yatra Visa Planner'!$A$4:$K$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Yatra Wishlist'!$A$4:$N$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Places Visited'!$A$4:$H$358</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Yatra Wishlist'!$A$4:$N$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -563,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -793,27 +795,27 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Wishlist ideas (open)</t>
+          <t>Places / sites logged (master list)</t>
         </is>
       </c>
       <c r="B18" s="6">
-        <f>COUNTIFS('Yatra Wishlist'!K5:K200,"&lt;&gt;Done",'Yatra Wishlist'!K5:K200,"&lt;&gt;Dropped",'Yatra Wishlist'!B5:B200,"&lt;&gt;")</f>
+        <f>'Places Visited'!$B$62</f>
         <v/>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>See Yatra Wishlist</t>
+          <t>See Places Visited</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Valid visas right now</t>
+          <t xml:space="preserve">  of which ISKCON / temples</t>
         </is>
       </c>
       <c r="B19" s="6">
-        <f>COUNTIF('Visas Held'!H5:H30,"VALID")</f>
+        <f>'Places Visited'!$B$63</f>
         <v/>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -821,81 +823,121 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
+          <t>Distinct cities logged</t>
+        </is>
+      </c>
+      <c r="B20" s="6">
+        <f>'Places Visited'!$B$64</f>
+        <v/>
+      </c>
+      <c r="C20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Wishlist ideas (open)</t>
+        </is>
+      </c>
+      <c r="B21" s="6">
+        <f>COUNTIFS('Yatra Wishlist'!K5:K200,"&lt;&gt;Done",'Yatra Wishlist'!K5:K200,"&lt;&gt;Dropped",'Yatra Wishlist'!B5:B200,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>See Yatra Wishlist</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Valid visas right now</t>
+        </is>
+      </c>
+      <c r="B22" s="6">
+        <f>COUNTIF('Visas Held'!H5:H30,"VALID")</f>
+        <v/>
+      </c>
+      <c r="C22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
           <t>Expired visas to renew</t>
         </is>
       </c>
-      <c r="B20" s="6">
+      <c r="B23" s="6">
         <f>COUNTIF('Visas Held'!H5:H30,"EXPIRED")</f>
         <v/>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Schengen &amp; UK</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Top actions</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="48" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>Passport expires 17 Sep 2028</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Most countries need 6 months validity -&gt; practical last safe travel date ~17 Mar 2028. Start renewal ~Sep 2027. Passports issued in India are e-passports since 28 May 2025. Keep old passport: US &amp; Australia visas stay valid but must be carried; tell Australia Home Affairs new passport number (ImmiAccount).</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="48" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>Schengen: no valid visa</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Both France visas expired (Apr 2026). You now have 2 lawful visas in 3 years -&gt; eligible for the EU 'cascade' 2-year multiple-entry visa. Apply 3 months before the next Europe yatra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="48" customHeight="1">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>UK: no valid visa</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>UK visa expired 29 Dec 2024. Apply 3-4 weeks ahead; consider a 2-year or 5-year Standard Visitor visa if you will return often.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>Australia: confirm stream</t>
+          <t>Passport expires 17 Sep 2028</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Visa is Business Visitor stream (condition 8115). A pilgrimage yatra with devotees may count as tourism - confirm whether to apply for a Tourist-stream visa.</t>
+          <t>Most countries need 6 months validity -&gt; practical last safe travel date ~17 Mar 2028. Start renewal ~Sep 2027. Passports issued in India are e-passports since 28 May 2025. Keep old passport: US &amp; Australia visas stay valid but must be carried; tell Australia Home Affairs new passport number (ImmiAccount).</t>
         </is>
       </c>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
+          <t>Schengen: no valid visa</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Both France visas expired (Apr 2026). You now have 2 lawful visas in 3 years -&gt; eligible for the EU 'cascade' 2-year multiple-entry visa. Apply 3 months before the next Europe yatra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>UK: no valid visa</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>UK visa expired 29 Dec 2024. Apply 3-4 weeks ahead; consider a 2-year or 5-year Standard Visitor visa if you will return often.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Australia: confirm stream</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Visa is Business Visitor stream (condition 8115). A pilgrimage yatra with devotees may count as tourism - confirm whether to apply for a Tourist-stream visa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
           <t>Malaysia visa-free ends 31 Dec 2026</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>Get visa/e-visa for any 2027 Malaysia yatra unless extended.</t>
         </is>
@@ -907,6 +949,371 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001F2A44"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Trips in your dashboard with NO passport stamp yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Your spreadsheet shows these; the passport scan (to Nov 2025) doesn't. Confirm -&gt; copy to Travel Log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Trip</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Where recorded</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed? (Y/N)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Europe (Schengen)</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>45934</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>45947</v>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard 'MKCD' column</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Schengen visa #2 only valid from 21 Oct 2025 - this window pre-dates it; likely moved to Nov</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="G5" s="19" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Europe (Schengen)</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>45967</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>45981</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard 'MKCD' column</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Inside Schengen #2 validity (21 Oct 2025-19 Apr 2026); no stamp in Nov-2025 scan</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="G6" s="19" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Sri Lanka (Ramayan Yatra)</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>46040</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>46048</v>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard 'MKCD' column</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Future relative to scan; confirm if done</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="G7" s="19" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Australia (Yatra)</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>46063</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>46072</v>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard 'MKCD' column</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Visa granted 13 Nov 2025; would be FIRST Australia entry - confirm</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="G8" s="19" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Bali, Indonesia</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>46074</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>46080</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard 'MKCD' column</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Nepal (Muktinath Yatra)</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>45592</v>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>45598</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard yatra column</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>No 2024 Nepal stamp seen - may have been an escorted group yatra or not run</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Sri Lanka (Ramayan Yatra)</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="n">
+        <v>45627</v>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>45633</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard yatra column</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>No Dec-2024 SL stamp in scan - confirm</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="G11" s="19" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Thailand / Cambodia Yatra</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>45664</v>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>45669</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard yatra column</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>No Jan-2025 stamp in scan - confirm</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Nepal (Muktinath Yatra)</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="n">
+        <v>45748</v>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>45768</v>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard yatra column</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>No Apr-2025 stamp in scan - confirm</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>OOS / BJ (domestic?)</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="n">
+        <v>45727</v>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>45732</v>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard 'MKCD' column</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Label unclear ('OOS'); probably out-of-station, not international</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Ignore?</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001F2A44"/>
@@ -1102,7 +1509,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001F2A44"/>
@@ -1874,7 +2281,7 @@
         <v>45488</v>
       </c>
       <c r="D16" s="12" t="n">
-        <v>45500</v>
+        <v>45491</v>
       </c>
       <c r="E16" s="9">
         <f>IF(AND(ISNUMBER(C16),ISNUMBER(D16)),D16-C16+1,"")</f>
@@ -1892,7 +2299,7 @@
       </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
-          <t>Milan Malpensa (Italy)</t>
+          <t>By road to Brussels</t>
         </is>
       </c>
       <c r="I16" s="9" t="inlineStr">
@@ -1912,7 +2319,7 @@
       </c>
       <c r="L16" s="9" t="inlineStr">
         <is>
-          <t>Schengen trip 15-27 Jul 2024 covering France, Belgium, Netherlands, Germany, Switzerland, Italy/Rome, Vatican City; France dates = whole-trip window, split per country when known</t>
+          <t>Paris 15-17 Jul (Seine, Eiffel, Louvre), ISKCON New Mayapur 17 Jul; left for Brussels 18 Jul. Dates inferred from itinerary Days 4-7 anchored on CDG stamp</t>
         </is>
       </c>
     </row>
@@ -1925,8 +2332,12 @@
           <t>Belgium</t>
         </is>
       </c>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
+      <c r="C17" s="10" t="n">
+        <v>45491</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>45492</v>
+      </c>
       <c r="E17" s="9">
         <f>IF(AND(ISNUMBER(C17),ISNUMBER(D17)),D17-C17+1,"")</f>
         <v/>
@@ -1938,12 +2349,12 @@
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>By road/rail within Schengen (no stamp)</t>
+          <t>By road from Paris</t>
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>By road/rail within Schengen (no stamp)</t>
+          <t>By road to Amsterdam</t>
         </is>
       </c>
       <c r="I17" s="9" t="inlineStr">
@@ -1953,7 +2364,7 @@
       </c>
       <c r="J17" s="9" t="inlineStr">
         <is>
-          <t>Your confirmation (Oct 2026): visited during the 15-27 Jul 2024 Europe trip</t>
+          <t>Itinerary Day 7: Brussels + ISKCON Radhadesh; dates inferred</t>
         </is>
       </c>
       <c r="K17" s="11" t="inlineStr">
@@ -1963,7 +2374,7 @@
       </c>
       <c r="L17" s="9" t="inlineStr">
         <is>
-          <t>Dates unknown - within 15-27 Jul 2024; add from itinerary</t>
+          <t>Brussels Grand Place, Manneken Pis, Radhadesh (Durbuy)</t>
         </is>
       </c>
     </row>
@@ -1976,8 +2387,12 @@
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
+      <c r="C18" s="10" t="n">
+        <v>45492</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>45493</v>
+      </c>
       <c r="E18" s="9">
         <f>IF(AND(ISNUMBER(C18),ISNUMBER(D18)),D18-C18+1,"")</f>
         <v/>
@@ -1989,12 +2404,12 @@
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>By road/rail within Schengen (no stamp)</t>
+          <t>By road from Brussels</t>
         </is>
       </c>
       <c r="H18" s="9" t="inlineStr">
         <is>
-          <t>By road/rail within Schengen (no stamp)</t>
+          <t>By road to Cologne</t>
         </is>
       </c>
       <c r="I18" s="9" t="inlineStr">
@@ -2004,7 +2419,7 @@
       </c>
       <c r="J18" s="9" t="inlineStr">
         <is>
-          <t>Your confirmation (Oct 2026): visited during the 15-27 Jul 2024 Europe trip</t>
+          <t>Itinerary Days 8-9: Amsterdam canal cruise + city; dates inferred</t>
         </is>
       </c>
       <c r="K18" s="11" t="inlineStr">
@@ -2014,7 +2429,7 @@
       </c>
       <c r="L18" s="9" t="inlineStr">
         <is>
-          <t>Dates unknown - within 15-27 Jul 2024; add from itinerary</t>
+          <t>Amsterdam; 'Hare Krishna Valley' temple on Day 9 (confirm which)</t>
         </is>
       </c>
     </row>
@@ -2027,8 +2442,12 @@
           <t>Germany</t>
         </is>
       </c>
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
+      <c r="C19" s="10" t="n">
+        <v>45493</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>45494</v>
+      </c>
       <c r="E19" s="9">
         <f>IF(AND(ISNUMBER(C19),ISNUMBER(D19)),D19-C19+1,"")</f>
         <v/>
@@ -2040,12 +2459,12 @@
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>By road/rail within Schengen (no stamp)</t>
+          <t>By road from Amsterdam</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>By road/rail within Schengen (no stamp)</t>
+          <t>By road via Rhine Falls to Zurich</t>
         </is>
       </c>
       <c r="I19" s="9" t="inlineStr">
@@ -2055,7 +2474,7 @@
       </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
-          <t>Your confirmation (Oct 2026): visited during the 15-27 Jul 2024 Europe trip</t>
+          <t>Itinerary Days 9-10: Cologne, Black Forest, Triberg; dates inferred</t>
         </is>
       </c>
       <c r="K19" s="11" t="inlineStr">
@@ -2063,11 +2482,7 @@
           <t>Check</t>
         </is>
       </c>
-      <c r="L19" s="9" t="inlineStr">
-        <is>
-          <t>Dates unknown - within 15-27 Jul 2024; add from itinerary</t>
-        </is>
-      </c>
+      <c r="L19" s="9" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="n">
@@ -2078,8 +2493,12 @@
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
+      <c r="C20" s="10" t="n">
+        <v>45494</v>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>45496</v>
+      </c>
       <c r="E20" s="9">
         <f>IF(AND(ISNUMBER(C20),ISNUMBER(D20)),D20-C20+1,"")</f>
         <v/>
@@ -2091,12 +2510,12 @@
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>By road/rail within Schengen (no stamp)</t>
+          <t>Rhine Falls (by road)</t>
         </is>
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>By road/rail within Schengen (no stamp)</t>
+          <t>By road to Milan</t>
         </is>
       </c>
       <c r="I20" s="9" t="inlineStr">
@@ -2106,7 +2525,7 @@
       </c>
       <c r="J20" s="9" t="inlineStr">
         <is>
-          <t>Your confirmation (Oct 2026): visited during the 15-27 Jul 2024 Europe trip</t>
+          <t>Itinerary Days 10-12: Rhine Falls, Zurich, Lucerne, Mt Titlis; dates inferred</t>
         </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
@@ -2114,11 +2533,7 @@
           <t>Check</t>
         </is>
       </c>
-      <c r="L20" s="9" t="inlineStr">
-        <is>
-          <t>Dates unknown - within 15-27 Jul 2024; add from itinerary</t>
-        </is>
-      </c>
+      <c r="L20" s="9" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="n">
@@ -2129,8 +2544,12 @@
           <t>Vatican City</t>
         </is>
       </c>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n"/>
+      <c r="C21" s="10" t="n">
+        <v>45499</v>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>45499</v>
+      </c>
       <c r="E21" s="9">
         <f>IF(AND(ISNUMBER(C21),ISNUMBER(D21)),D21-C21+1,"")</f>
         <v/>
@@ -2147,17 +2566,17 @@
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>On foot from Rome (no border control)</t>
+          <t>On foot from Rome</t>
         </is>
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Schengen C visa #1 (Vatican has open border with Italy)</t>
+          <t>Schengen C visa #1 (open border with Italy)</t>
         </is>
       </c>
       <c r="J21" s="9" t="inlineStr">
         <is>
-          <t>Your confirmation (Oct 2026): visited from Rome during the 15-27 Jul 2024 Europe trip</t>
+          <t>Itinerary Day 15: St Peter's Square &amp; Basilica; date inferred</t>
         </is>
       </c>
       <c r="K21" s="11" t="inlineStr">
@@ -2167,7 +2586,7 @@
       </c>
       <c r="L21" s="9" t="inlineStr">
         <is>
-          <t>Sovereign state; same day(s) as Rome - add date from itinerary</t>
+          <t>Same day as Rome</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2599,9 @@
           <t>Italy</t>
         </is>
       </c>
-      <c r="C22" s="10" t="n"/>
+      <c r="C22" s="10" t="n">
+        <v>45496</v>
+      </c>
       <c r="D22" s="10" t="n">
         <v>45500</v>
       </c>
@@ -2195,7 +2616,7 @@
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>By road/rail within Schengen (Rome visited)</t>
+          <t>By road from Lucerne</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">
@@ -2210,7 +2631,7 @@
       </c>
       <c r="J22" s="9" t="inlineStr">
         <is>
-          <t>Your confirmation (Oct 2026): Rome visited; Passport p.17: Malpensa exit stamp 27 Jul 2024</t>
+          <t>Itinerary Days 12-16: Milan, Padova, Venice, Arezzo, Florence, Pisa, Rome; Malpensa exit stamp 27 Jul 2024</t>
         </is>
       </c>
       <c r="K22" s="11" t="inlineStr">
@@ -2220,7 +2641,7 @@
       </c>
       <c r="L22" s="9" t="inlineStr">
         <is>
-          <t>Entry date unknown - within 15-27 Jul 2024; departed Schengen from Milan</t>
+          <t>Entry date inferred; exit stamped</t>
         </is>
       </c>
     </row>
@@ -2233,10 +2654,12 @@
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="C23" s="12" t="n">
+      <c r="C23" s="10" t="n">
         <v>45500</v>
       </c>
-      <c r="D23" s="10" t="n"/>
+      <c r="D23" s="10" t="n">
+        <v>45504</v>
+      </c>
       <c r="E23" s="9">
         <f>IF(AND(ISNUMBER(C23),ISNUMBER(D23)),D23-C23+1,"")</f>
         <v/>
@@ -2253,7 +2676,7 @@
       </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
-          <t>(UK does not stamp exit)</t>
+          <t>London -&gt; Dubai (UK does not stamp exit)</t>
         </is>
       </c>
       <c r="I23" s="9" t="inlineStr">
@@ -2263,17 +2686,17 @@
       </c>
       <c r="J23" s="9" t="inlineStr">
         <is>
-          <t>Passport p.23: Gatwick stamp 27 Jul 2024</t>
-        </is>
-      </c>
-      <c r="K23" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>Passport p.23: Gatwick stamp 27 Jul 2024; UAE entry 1 Aug 2024 -&gt; UK exit ~31 Jul (inferred)</t>
+        </is>
+      </c>
+      <c r="K23" s="11" t="inlineStr">
+        <is>
+          <t>Check</t>
         </is>
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Left UK by 01 Aug 2024 (UAE entry)</t>
+          <t>London (itinerary Days 1-3 done AFTER the continent): Bhaktivedanta Manor, city tour, London Eye, Thames cruise, Madame Tussauds</t>
         </is>
       </c>
     </row>
@@ -2848,7 +3271,7 @@
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Schengen C visa #1 (Vatican has open border with Italy)</t>
+          <t>Schengen C visa #1 (open border with Italy)</t>
         </is>
       </c>
     </row>
@@ -7858,6 +8281,2157 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H64"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Places Visited - MASTER list of cities &amp; sites already covered</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Keep adding rows (one per site). Country Summary counts countries; this sheet counts cities and places. Rows saying 'if visited' / 'confirm' are guesses - delete or confirm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>City / area</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Place / site</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Date / trip</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Arrival London (Gatwick)</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Transit hub</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>27 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>Gatwick stamp 27 Jul 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Watford (Aldenham)</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Bhaktivedanta Manor - Hare Krishna Temple</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>ISKCON/Temple</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>27 Jul-1 Aug 2024</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>Prabhupada's UK centre, donated by George Harrison</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Tower of London</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>27 Jul-1 Aug 2024</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>St Paul's Cathedral</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>27 Jul-1 Aug 2024</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Buckingham Palace - Changing of the Guard</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>27 Jul-1 Aug 2024</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>London Eye</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>27 Jul-1 Aug 2024</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>River Thames cruise</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Cruise/Ride</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>27 Jul-1 Aug 2024</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Madame Tussauds</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Museum</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>27 Jul-1 Aug 2024</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>London Bridge / Tower Bridge area</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>27 Jul-1 Aug 2024</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Big Ben &amp; Houses of Parliament (viewed)</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>27 Jul-1 Aug 2024</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Seen from London Eye / cruise</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Arrival Paris CDG</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Transit hub</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>15 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>CDG stamp 15 Jul 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Seine River cruise</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Cruise/Ride</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>15 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Eiffel Tower (2nd floor)</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>16 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Louvre Museum (Mona Lisa, Venus de Milo)</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Museum</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>16 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Arc de Triomphe, Champs-Elysees, Place de la Concorde</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>City tour</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>16 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Montmartre, Latin Quarter, Le Marais</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>City tour</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>16 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Notre-Dame (viewed from Seine)</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>15 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Lucay-le-Male (Indre)</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>ISKCON New Mayapur (Nouvelle Mayapura)</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>ISKCON/Temple</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>17 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Itinerary calls it 'outskirts of Paris'; it is ~250 km south</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>ISKCON Paris (Sarcelles) - if visited</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>ISKCON/Temple</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>15-17 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Not in itinerary - delete if not visited</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Brussels</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Grand Place &amp; Town Hall</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>18 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Brussels</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Manneken Pis</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>18 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H25" s="9" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Durbuy (Septon)</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>ISKCON Radhadesh (Chateau de Petite Somme)</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>ISKCON/Temple</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>18 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>Bhaktivedanta College campus, Ardennes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Canal cruise</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>Cruise/Ride</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>19 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Dam Square &amp; Royal Palace</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>19 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>Anne Frank House (exterior)</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>19 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Jordaan district</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>City tour</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>19 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Netherlands / Germany</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>(countryside)</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>'Hare Krishna Valley' temple (per itinerary)</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>ISKCON/Temple</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>20 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>Itinerary name is vague - confirm which temple (e.g. ISKCON Amsterdam, Simhachalam/Germany, Goloka Dhama/Abentheuer). Edit country when known.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>Cologne Cathedral &amp; Old Town</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>20 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>Black Forest</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>Black Forest drive</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>21 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H33" s="9" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Triberg</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>Triberg - cuckoo clock shop (and falls area)</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>21 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H34" s="9" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Neuhausen am Rheinfall</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>Rhine Falls (Europe's largest waterfall)</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>21 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H35" s="9" t="inlineStr">
+        <is>
+          <t>Swiss side of the German border</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Zurich</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>Zurich Old Town</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>City tour</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>21 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H36" s="9" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>Lucerne</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>Chapel Bridge, Water Tower, Lake Lucerne, Old Town</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr">
+        <is>
+          <t>22 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H37" s="9" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>Engelberg</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>Mt Titlis - Rotair cable car, Cliff Walk, Ice Flyer</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>22 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H38" s="9" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>Zurich</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>ISKCON Zurich (Krishna Tempel) - if visited</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>ISKCON/Temple</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>21-22 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="inlineStr">
+        <is>
+          <t>Not in itinerary - delete if not visited</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Milan</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>Villaggio Hare Krishna (Chignolo d'Isola)</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>ISKCON/Temple</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>23 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G40" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H40" s="9" t="inlineStr">
+        <is>
+          <t>ISKCON Milan farm community</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>Milan</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>Duomo di Milano, Galleria Vittorio Emanuele II, Sforza Castle, Brera</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>City tour</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>23 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H41" s="9" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Padova</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>Padova (overnight base)</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>City tour</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>24 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H42" s="9" t="inlineStr">
+        <is>
+          <t>Prato della Valle / St Anthony basilica if seen</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>Venice</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>Gondola ride</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>Cruise/Ride</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>24 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H43" s="9" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>Venice</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>St Mark's Square, Doge's Palace, Rialto Bridge</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="inlineStr">
+        <is>
+          <t>24 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G44" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H44" s="9" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Arezzo</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>Arezzo (overnight base)</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>City tour</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>25 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Florence</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>Florence Cathedral (Duomo), Ponte Vecchio, Piazza della Signoria</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>25 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H46" s="9" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>Leaning Tower of Pisa</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>25 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Florence</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>ISKCON Florence (Villa Vrindavana, San Casciano)</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>ISKCON/Temple</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>25 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>Rome</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>Colosseum (outside), Roman Forum, Pantheon</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>26 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H49" s="9" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>Milan</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>Departure Milan Malpensa</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>Transit hub</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>27 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H50" s="9" t="inlineStr">
+        <is>
+          <t>Malpensa stamp 27 Jul 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>Vatican City</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>Vatican City</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>St Peter's Square &amp; St Peter's Basilica</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>26 Jul 2024</t>
+        </is>
+      </c>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>Europe+London yatra, Jul 2024 (itinerary + passport stamps)</t>
+        </is>
+      </c>
+      <c r="H51" s="9" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>Sri Lanka</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>Colombo (BIA)</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t>Colombo - Ramayana trail bases</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>City tour</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>Sep-Oct 2019; Dec 2019; Jan 2022</t>
+        </is>
+      </c>
+      <c r="G52" s="9" t="inlineStr">
+        <is>
+          <t>Passport stamps</t>
+        </is>
+      </c>
+      <c r="H52" s="9" t="inlineStr">
+        <is>
+          <t>Add sites visited (e.g. Seetha Amman Kovil, Ashok Vatika, Munneswaram, Kelaniya)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>Kathmandu</t>
+        </is>
+      </c>
+      <c r="D53" s="11" t="inlineStr">
+        <is>
+          <t>Kathmandu (Pashupatinath etc.)</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>City tour</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>May 2019; Apr 2022 (+Mar 2019 exit)</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>Passport stamps</t>
+        </is>
+      </c>
+      <c r="H53" s="9" t="inlineStr">
+        <is>
+          <t>Add sites (Pashupatinath, Budhanilkantha, Krishna Mandir Patan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>Pokhara / Jomsom / Muktinath</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>Muktinath yatra route</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t>ISKCON/Temple</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="inlineStr">
+        <is>
+          <t>(from your dashboard - confirm trip)</t>
+        </is>
+      </c>
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>Your dashboard</t>
+        </is>
+      </c>
+      <c r="H54" s="9" t="inlineStr">
+        <is>
+          <t>Add when confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>Bangkok (BKK)</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr">
+        <is>
+          <t>Bangkok</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>City tour</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>Feb 2023 (x2); Jun 2023</t>
+        </is>
+      </c>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>Passport stamps</t>
+        </is>
+      </c>
+      <c r="H55" s="9" t="inlineStr">
+        <is>
+          <t>Add sites (ISKCON Bangkok, Wat Arun, Grand Palace...)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>Cambodia</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>Siem Reap</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>Angkor Wat / Angkor Thom</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="inlineStr">
+        <is>
+          <t>Feb 2023; Jun 2023</t>
+        </is>
+      </c>
+      <c r="G56" s="9" t="inlineStr">
+        <is>
+          <t>Passport stamps (Siem Reap)</t>
+        </is>
+      </c>
+      <c r="H56" s="9" t="inlineStr">
+        <is>
+          <t>Confirm sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t>City tour</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="inlineStr">
+        <is>
+          <t>1-~5 Aug 2024</t>
+        </is>
+      </c>
+      <c r="G57" s="9" t="inlineStr">
+        <is>
+          <t>Passport stamp</t>
+        </is>
+      </c>
+      <c r="H57" s="9" t="inlineStr">
+        <is>
+          <t>Add sites (ISKCON Dubai Bur Dubai, Burj Khalifa...)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="B58" s="9" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>(cities to add)</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>USA trip Sep 2025</t>
+        </is>
+      </c>
+      <c r="E58" s="9" t="inlineStr">
+        <is>
+          <t>City tour</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="inlineStr">
+        <is>
+          <t>4-30 Sep 2025</t>
+        </is>
+      </c>
+      <c r="G58" s="9" t="inlineStr">
+        <is>
+          <t>Passport stamp</t>
+        </is>
+      </c>
+      <c r="H58" s="9" t="inlineStr">
+        <is>
+          <t>Add cities &amp; temples visited (27 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>Counts (auto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Places logged</t>
+        </is>
+      </c>
+      <c r="B62">
+        <f>COUNTA(D5:D358)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ISKCON / temples</t>
+        </is>
+      </c>
+      <c r="B63">
+        <f>COUNTIF(E5:E358,"ISKCON/Temple")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Distinct cities</t>
+        </is>
+      </c>
+      <c r="B64">
+        <f>SUMPRODUCT((C5:C58&lt;&gt;"")/COUNTIF(C5:C58,C5:C58&amp;""))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:H358"/>
+  <dataValidations count="1">
+    <dataValidation sqref="E5:E358" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ISKCON/Temple,Landmark,Museum,Nature,Cruise/Ride,City tour,Transit hub"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001F2A44"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8529,369 +11103,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="001F2A44"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Trips in your dashboard with NO passport stamp yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Your spreadsheet shows these; the passport scan (to Nov 2025) doesn't. Confirm -&gt; copy to Travel Log.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Trip</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>From</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>To</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Where recorded</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Observation</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Action</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Confirmed? (Y/N)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Europe (Schengen)</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="n">
-        <v>45934</v>
-      </c>
-      <c r="C5" s="12" t="n">
-        <v>45947</v>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>Dashboard 'MKCD' column</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr">
-        <is>
-          <t>Schengen visa #2 only valid from 21 Oct 2025 - this window pre-dates it; likely moved to Nov</t>
-        </is>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>Confirm</t>
-        </is>
-      </c>
-      <c r="G5" s="19" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Europe (Schengen)</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="n">
-        <v>45967</v>
-      </c>
-      <c r="C6" s="12" t="n">
-        <v>45981</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Dashboard 'MKCD' column</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>Inside Schengen #2 validity (21 Oct 2025-19 Apr 2026); no stamp in Nov-2025 scan</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>Confirm</t>
-        </is>
-      </c>
-      <c r="G6" s="19" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Sri Lanka (Ramayan Yatra)</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="n">
-        <v>46040</v>
-      </c>
-      <c r="C7" s="12" t="n">
-        <v>46048</v>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>Dashboard 'MKCD' column</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>Future relative to scan; confirm if done</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>Confirm</t>
-        </is>
-      </c>
-      <c r="G7" s="19" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>Australia (Yatra)</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="n">
-        <v>46063</v>
-      </c>
-      <c r="C8" s="12" t="n">
-        <v>46072</v>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>Dashboard 'MKCD' column</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>Visa granted 13 Nov 2025; would be FIRST Australia entry - confirm</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>Confirm</t>
-        </is>
-      </c>
-      <c r="G8" s="19" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>Bali, Indonesia</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="n">
-        <v>46074</v>
-      </c>
-      <c r="C9" s="12" t="n">
-        <v>46080</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Dashboard 'MKCD' column</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>Confirm</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Confirm</t>
-        </is>
-      </c>
-      <c r="G9" s="19" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>Nepal (Muktinath Yatra)</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="n">
-        <v>45592</v>
-      </c>
-      <c r="C10" s="12" t="n">
-        <v>45598</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Dashboard yatra column</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>No 2024 Nepal stamp seen - may have been an escorted group yatra or not run</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Confirm</t>
-        </is>
-      </c>
-      <c r="G10" s="19" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Sri Lanka (Ramayan Yatra)</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="n">
-        <v>45627</v>
-      </c>
-      <c r="C11" s="12" t="n">
-        <v>45633</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Dashboard yatra column</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>No Dec-2024 SL stamp in scan - confirm</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Confirm</t>
-        </is>
-      </c>
-      <c r="G11" s="19" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>Thailand / Cambodia Yatra</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="n">
-        <v>45664</v>
-      </c>
-      <c r="C12" s="12" t="n">
-        <v>45669</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Dashboard yatra column</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>No Jan-2025 stamp in scan - confirm</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Confirm</t>
-        </is>
-      </c>
-      <c r="G12" s="19" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Nepal (Muktinath Yatra)</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="n">
-        <v>45748</v>
-      </c>
-      <c r="C13" s="12" t="n">
-        <v>45768</v>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>Dashboard yatra column</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>No Apr-2025 stamp in scan - confirm</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>Confirm</t>
-        </is>
-      </c>
-      <c r="G13" s="19" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>OOS / BJ (domestic?)</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="n">
-        <v>45727</v>
-      </c>
-      <c r="C14" s="12" t="n">
-        <v>45732</v>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>Dashboard 'MKCD' column</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>Label unclear ('OOS'); probably out-of-station, not international</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>Ignore?</t>
-        </is>
-      </c>
-      <c r="G14" s="19" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add UAE tourist eVisa (Jul-Sep 2024) to visas held
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MuHAkrVAM6ipkG9EkAQkug
</commit_message>
<xml_diff>
--- a/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
+++ b/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>'Visas Held'!$B$14</f>
+        <f>'Visas Held'!$B$15</f>
         <v/>
       </c>
       <c r="C6" t="inlineStr">
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B7" s="6">
-        <f>'Visas Held'!$B$16</f>
+        <f>'Visas Held'!$B$17</f>
         <v/>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -669,7 +669,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>'Visas Held'!$B$17</f>
+        <f>'Visas Held'!$B$18</f>
         <v/>
       </c>
       <c r="C8" t="inlineStr">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>'Visas Held'!$B$18</f>
+        <f>'Visas Held'!$B$19</f>
         <v/>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -930,7 +930,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Schengen &amp; UK</t>
+          <t>Schengen, UK (UAE eVisa was single-use)</t>
         </is>
       </c>
     </row>
@@ -6319,12 +6319,12 @@
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>Visa/entry per stamp (Indian PP)</t>
+          <t>UAE Tourist eVisa, single entry, 30 days (issued Dubai 18 Jul 2024)</t>
         </is>
       </c>
       <c r="J24" s="9" t="inlineStr">
         <is>
-          <t>Passport p.10: UAE entry stamp 01 Aug 2024; India arrival RGI Hyderabad 05 Aug 2024</t>
+          <t>Passport p.10: UAE entry stamp 01 Aug 2024 + eVisa PDF; India arrival RGI Hyderabad 05 Aug 2024</t>
         </is>
       </c>
       <c r="K24" s="9" t="inlineStr">
@@ -7075,7 +7075,7 @@
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>Visa/entry per stamp (Indian PP)</t>
+          <t>UAE Tourist eVisa, single entry, 30 days (issued Dubai 18 Jul 2024)</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -7561,99 +7561,151 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>UAE Tourist eVisa</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Tourism - Single entry - 30 days (sponsor: Akbar Travels of India LLC)</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="n">
+        <v>45491</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>45550</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>30 days max stay</t>
+        </is>
+      </c>
+      <c r="H10" s="9">
+        <f>IF(E10&lt;TODAY(),"EXPIRED",IF(E10-TODAY()&lt;180,"EXPIRING SOON","VALID"))</f>
+        <v/>
+      </c>
+      <c r="I10" s="9">
+        <f>E10-TODAY()</f>
+        <v/>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>Used 1 Aug 2024 (Dubai); entry validity expired 15 Sep 2024</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr"/>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>eVisa PDF (entry permit 201/2024/...)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>PASSPORT</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Document</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Indian ordinary passport (36 pages)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Issued</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>43361</v>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Indian ordinary passport (36 pages)</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Expires</t>
+          <t>Issued</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>47013</v>
+        <v>43361</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Place of issue</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Hyderabad</t>
-        </is>
+          <t>Expires</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>47013</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Days to expiry</t>
-        </is>
-      </c>
-      <c r="B16" s="14">
-        <f>B14-TODAY()</f>
-        <v/>
+          <t>Place of issue</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>6-month rule date</t>
-        </is>
-      </c>
-      <c r="B17" s="5">
-        <f>EDATE(B14,-6)</f>
+          <t>Days to expiry</t>
+        </is>
+      </c>
+      <c r="B17" s="14">
+        <f>B15-TODAY()</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
+          <t>6-month rule date</t>
+        </is>
+      </c>
+      <c r="B18" s="5">
+        <f>EDATE(B15,-6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
           <t>Start renewal by</t>
         </is>
       </c>
-      <c r="B18" s="5">
-        <f>EDATE(B14,-12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="B19" s="5">
+        <f>EDATE(B15,-12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Old passport (issued 15/10/2008, Bangalore) not supplied - earlier travel not captured.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H5:H30">
+  <conditionalFormatting sqref="H5:H31">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"EXPIRED"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Add passport renewal, Schengen and UK visa renewal as next steps in Yatra Wishlist
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MuHAkrVAM6ipkG9EkAQkug
</commit_message>
<xml_diff>
--- a/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
+++ b/docs/visa-travel/MKCD_Visa_Travel_Tracker.xlsx
@@ -29,7 +29,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Yatra Visa Planner'!$A$4:$L$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Places Visited'!$A$4:$H$406</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'World Checklist'!$A$4:$I$831</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Yatra Wishlist'!$A$4:$N$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Yatra Wishlist'!$A$4:$N$116</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19811,7 +19811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -19922,42 +19922,42 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Mysore Dasara</t>
+          <t>NEXT STEP 1: Schengen multi-entry visa (2-yr -&gt; 5-yr)</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Mysuru, Karnataka, India</t>
+          <t>Apply via VFS (France/Germany/Switzerland), India</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Festival yatra</t>
+          <t>Visa renewal - #1 priority</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>Sep-Oct (Navaratri)</t>
+          <t>Apply 3 months before next Europe yatra; passport renewal first if aiming for 5-yr</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>10 days ending Vijayadashami; Jamboo Savari on the last day</t>
+          <t>EU cascade: 2 lawful Schengen visas in 3 yrs -&gt; 2-yr MEV; 5-yr needs ~5.5 yrs passport validity (yours ends Sep 2028)</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>None (domestic)</t>
+          <t>EUR 90 + VFS fee; 15-45 days processing; docs: both used visas (Jul 2024, Oct 2025-Apr 2026), itinerary/invitation from ISKCON Europe, funds, insurance</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t>Palace illumination, Chamundi Hill, Jamboo Savari procession. Book stay months ahead; ISKCON Mysore nearby. Combine with Srirangapatna, Melukote.</t>
+          <t>Single biggest reach gain (~65 destinations). Prefer German/Swiss-issued if Singapore 96-h transit matters. Ask explicitly for 'multiple entry, long validity'.</t>
         </is>
       </c>
       <c r="J5" s="22" t="inlineStr">
@@ -19967,7 +19967,7 @@
       </c>
       <c r="K5" s="22" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="L5" s="22" t="inlineStr"/>
@@ -19982,42 +19982,42 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Tirupati Balaji Brahmotsavam</t>
+          <t>NEXT STEP 2: UK Standard Visitor visa (2-yr or 5-yr)</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Tirumala, Andhra Pradesh, India</t>
+          <t>Apply online gov.uk + VFS biometrics, India</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Festival yatra</t>
+          <t>Visa renewal - #2 priority</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Sep-Oct (Salakatla Brahmotsavam); some years a 2nd Navaratri Brahmotsavam</t>
+          <t>Apply 4-6 weeks before next UK yatra (Bhaktivedanta Manor)</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>9 days; Garuda Seva day is the peak</t>
+          <t>Fees from 8 Apr 2026: GBP 135 (6-mo) / 506 (2-yr) / 903 (5-yr) / 1,128 (10-yr); max 6 months per visit</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>None; TTD darshan tokens / SED booking via tirupatibalaji.ap.gov.in</t>
+          <t>GBP 506-903; ~3 weeks; previous UK visa (Jun-Dec 2024, used) helps</t>
         </is>
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Vahana sevas each morning/evening; Garuda Seva night draws lakhs. Arrange accommodation via TTD or HKM contacts well in advance.</t>
+          <t>Also covers Ireland via BIVS (enter UK first). Gibraltar via UK visa ended 15 Jul 2026. Not ETA-eligible.</t>
         </is>
       </c>
       <c r="J6" s="22" t="inlineStr">
@@ -20027,7 +20027,7 @@
       </c>
       <c r="K6" s="22" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="L6" s="22" t="inlineStr"/>
@@ -20042,42 +20042,42 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Vaishno Devi</t>
+          <t>NEXT STEP 0: Indian passport renewal</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Katra, Jammu &amp; Kashmir, India</t>
+          <t>Passport Seva Kendra, Hyderabad</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>Shakti-peetha trek</t>
+          <t>Pre-requisite</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Mar-Jun and Sep-Nov (avoid peak summer rush and Jan snow)</t>
+          <t>Start by Sep 2027 at latest; earlier (2026-27) if applying for 5-yr Schengen</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Navaratri very crowded</t>
+          <t>Current passport expires 17 Sep 2028; 6-month rule bites from Mar 2028</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>3-4 (with travel)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>None; free RFID yatra card from SMVDSB (online or Katra)</t>
+          <t>Rs 1,500 (36 pp) / 2,000 (60 pp); e-passport issued since May 2025</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>13 km trek from Katra (ponies/palki/helicopter available). Combine with Jammu Raghunath temple; optionally Amritsar.</t>
+          <t>Carry OLD passport with US &amp; Australia visas; update Australia Home Affairs (ImmiAccount) with new passport number.</t>
         </is>
       </c>
       <c r="J7" s="22" t="inlineStr">
@@ -20087,7 +20087,7 @@
       </c>
       <c r="K7" s="22" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="L7" s="22" t="inlineStr"/>
@@ -20102,42 +20102,42 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Amarnath Yatra</t>
+          <t>Mysore Dasara</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Pahalgam / Baltal, Jammu &amp; Kashmir, India</t>
+          <t>Mysuru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>High-altitude cave pilgrimage</t>
+          <t>Festival yatra</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>Jul-Aug only (yatra window set yearly by SASB)</t>
+          <t>Sep-Oct (Navaratri)</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>~45-60 days, Ashadha Purnima to Shravana Purnima (Raksha Bandhan)</t>
+          <t>10 days ending Vijayadashami; Jamboo Savari on the last day</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>Compulsory SASB registration + Compulsory Health Certificate from authorised doctor; RFID card; age 13-70</t>
+          <t>None (domestic)</t>
         </is>
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>Register as soon as the window opens (Mar-Apr). Pahalgam route 32 km (3 days) or Baltal 14 km (1 day); helicopter options. Needs fitness prep.</t>
+          <t>Palace illumination, Chamundi Hill, Jamboo Savari procession. Book stay months ahead; ISKCON Mysore nearby. Combine with Srirangapatna, Melukote.</t>
         </is>
       </c>
       <c r="J8" s="22" t="inlineStr">
@@ -20162,47 +20162,47 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Seven Sisters (North-East India)</t>
+          <t>Tirupati Balaji Brahmotsavam</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Assam, Meghalaya, Arunachal, Nagaland, Manipur, Mizoram, Tripura</t>
+          <t>Tirumala, Andhra Pradesh, India</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Multi-state exploration yatra</t>
+          <t>Festival yatra</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Oct-Apr (dry, clear)</t>
+          <t>Sep-Oct (Salakatla Brahmotsavam); some years a 2nd Navaratri Brahmotsavam</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Avoid Jun-Sep monsoon</t>
+          <t>9 days; Garuda Seva day is the peak</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>10-14</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>Inner Line Permit (ILP) for Arunachal, Nagaland, Mizoram, Manipur - online; none for Assam/Meghalaya/Tripura</t>
+          <t>None; TTD darshan tokens / SED booking via tirupatibalaji.ap.gov.in</t>
         </is>
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>Kamakhya (Guwahati), Majuli satras (Vaishnava), Tawang monastery, Cherrapunji/Living root bridges, Loktak lake, Tripureshwari temple. Plan as 2 circuits (Assam-Meghalaya-Arunachal; Manipur-Mizoram-Tripura-Nagaland).</t>
+          <t>Vahana sevas each morning/evening; Garuda Seva night draws lakhs. Arrange accommodation via TTD or HKM contacts well in advance.</t>
         </is>
       </c>
       <c r="J9" s="22" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K9" s="22" t="inlineStr">
@@ -20222,47 +20222,47 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Vaishno Devi</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Katra, Jammu &amp; Kashmir, India</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>City + temple exploration</t>
+          <t>Shakti-peetha trek</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Oct-Feb (pleasant); Ganesh Chaturthi (Aug-Sep) for the festival</t>
+          <t>Mar-Jun and Sep-Nov (avoid peak summer rush and Jan snow)</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Ganeshotsav 10 days ending Anant Chaturdashi</t>
+          <t>Navaratri very crowded</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>3-4 (with travel)</t>
         </is>
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>None (domestic)</t>
+          <t>None; free RFID yatra card from SMVDSB (online or Katra)</t>
         </is>
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>ISKCON NVCC (Katraj) and ISKCON Camp; Dagdusheth Halwai Ganapati; Alandi (Dnyaneshwar samadhi) and Dehu (Tukaram) - Warkari heritage; Jejuri Khandoba; Bhimashankar Jyotirlinga day trip; Shaniwar Wada, Parvati hill. Can combine with Pandharpur (Ashadhi Ekadashi) or Shirdi.</t>
+          <t>13 km trek from Katra (ponies/palki/helicopter available). Combine with Jammu Raghunath temple; optionally Amritsar.</t>
         </is>
       </c>
       <c r="J10" s="22" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K10" s="22" t="inlineStr">
@@ -20282,27 +20282,27 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Indore &amp; Madhya Pradesh</t>
+          <t>Amarnath Yatra</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Indore / Ujjain / Omkareshwar / Maheshwar, Madhya Pradesh, India</t>
+          <t>Pahalgam / Baltal, Jammu &amp; Kashmir, India</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Jyotirlinga + heritage yatra</t>
+          <t>High-altitude cave pilgrimage</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Oct-Mar (avoid Apr-Jun heat)</t>
+          <t>Jul-Aug only (yatra window set yearly by SASB)</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Ujjain Simhastha Kumbh next due 2028 (Apr-May); Mahakal Bhasma Aarti daily at ~4 am (book online)</t>
+          <t>~45-60 days, Ashadha Purnima to Shravana Purnima (Raksha Bandhan)</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
@@ -20312,12 +20312,12 @@
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>None (domestic); Bhasma Aarti permission via shrimahakaleshwar.com</t>
+          <t>Compulsory SASB registration + Compulsory Health Certificate from authorised doctor; RFID card; age 13-70</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Base at Indore (Khajrana Ganesh, ISKCON Indore, Sarafa night food street). Ujjain: Mahakaleshwar + Mahakal Lok corridor, Kal Bhairav, Sandipani Ashram (Krishna's school). Omkareshwar Jyotirlinga + parikrama; Maheshwar ghats (Ahilyabai); Mandu. Optional extension: Chitrakoot / Khajuraho / Sanchi. Plan a 2028 Simhastha batch separately.</t>
+          <t>Register as soon as the window opens (Mar-Apr). Pahalgam route 32 km (3 days) or Baltal 14 km (1 day); helicopter options. Needs fitness prep.</t>
         </is>
       </c>
       <c r="J11" s="22" t="inlineStr">
@@ -20342,42 +20342,42 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Mumbai - NMACC (Nita Mukesh Ambani Cultural Centre)</t>
+          <t>Seven Sisters (North-East India)</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>BKC, Mumbai, Maharashtra, India</t>
+          <t>Assam, Meghalaya, Arunachal, Nagaland, Manipur, Mizoram, Tripura</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Culture + temple exploration</t>
+          <t>Multi-state exploration yatra</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>Oct-Feb (dry season); check NMACC programme calendar for shows/exhibitions</t>
+          <t>Oct-Apr (dry, clear)</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Year-round; 'Swadesh' crafts exhibition is permanent, theatre shows are ticketed</t>
+          <t>Avoid Jun-Sep monsoon</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>10-14</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>None (domestic); NMACC show tickets via nmacc.com / BookMyShow</t>
+          <t>Inner Line Permit (ILP) for Arunachal, Nagaland, Mizoram, Manipur - online; none for Assam/Meghalaya/Tripura</t>
         </is>
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>NMACC: Grand Theatre, Studio Theatre, Cube, Art House exhibitions, Swadesh artisan showcase. Combine with ISKCON Juhu (Prabhupada samadhi/museum), ISKCON Chowpatty (Radha Gopinath), Siddhivinayak, Mahalakshmi, Babulnath, Mumba Devi; Elephanta caves day trip. Was already on your Bucket List tab.</t>
+          <t>Kamakhya (Guwahati), Majuli satras (Vaishnava), Tawang monastery, Cherrapunji/Living root bridges, Loktak lake, Tripureshwari temple. Plan as 2 circuits (Assam-Meghalaya-Arunachal; Manipur-Mizoram-Tripura-Nagaland).</t>
         </is>
       </c>
       <c r="J12" s="22" t="inlineStr">
@@ -20402,42 +20402,42 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Kerala</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Kerala, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>Temple + culture yatra</t>
+          <t>City + temple exploration</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>Oct-Mar; Sabarimala season Nov-Jan</t>
+          <t>Oct-Feb (pleasant); Ganesh Chaturthi (Aug-Sep) for the festival</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>Guruvayur Ekadasi (Nov-Dec); Thrissur Pooram (Apr-May)</t>
+          <t>Ganeshotsav 10 days ending Anant Chaturdashi</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>6-8</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>None (domestic); Sabarimala needs virtual-queue booking</t>
+          <t>None (domestic)</t>
         </is>
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Guruvayur, Padmanabhaswamy (dress code), Sabarimala, Ambalappuzha, Aranmula, Chottanikkara; backwaters. Combine with Kanyakumari/Suchindram.</t>
+          <t>ISKCON NVCC (Katraj) and ISKCON Camp; Dagdusheth Halwai Ganapati; Alandi (Dnyaneshwar samadhi) and Dehu (Tukaram) - Warkari heritage; Jejuri Khandoba; Bhimashankar Jyotirlinga day trip; Shaniwar Wada, Parvati hill. Can combine with Pandharpur (Ashadhi Ekadashi) or Shirdi.</t>
         </is>
       </c>
       <c r="J13" s="22" t="inlineStr">
@@ -20456,9 +20456,189 @@
         <v>46316</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Indore &amp; Madhya Pradesh</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Indore / Ujjain / Omkareshwar / Maheshwar, Madhya Pradesh, India</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Jyotirlinga + heritage yatra</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Oct-Mar (avoid Apr-Jun heat)</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Ujjain Simhastha Kumbh next due 2028 (Apr-May); Mahakal Bhasma Aarti daily at ~4 am (book online)</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>None (domestic); Bhasma Aarti permission via shrimahakaleshwar.com</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>Base at Indore (Khajrana Ganesh, ISKCON Indore, Sarafa night food street). Ujjain: Mahakaleshwar + Mahakal Lok corridor, Kal Bhairav, Sandipani Ashram (Krishna's school). Omkareshwar Jyotirlinga + parikrama; Maheshwar ghats (Ahilyabai); Mandu. Optional extension: Chitrakoot / Khajuraho / Sanchi. Plan a 2028 Simhastha batch separately.</t>
+        </is>
+      </c>
+      <c r="J14" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K14" s="22" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="L14" s="22" t="inlineStr"/>
+      <c r="M14" s="22" t="inlineStr"/>
+      <c r="N14" s="12" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Mumbai - NMACC (Nita Mukesh Ambani Cultural Centre)</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>BKC, Mumbai, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Culture + temple exploration</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Oct-Feb (dry season); check NMACC programme calendar for shows/exhibitions</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Year-round; 'Swadesh' crafts exhibition is permanent, theatre shows are ticketed</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>None (domestic); NMACC show tickets via nmacc.com / BookMyShow</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>NMACC: Grand Theatre, Studio Theatre, Cube, Art House exhibitions, Swadesh artisan showcase. Combine with ISKCON Juhu (Prabhupada samadhi/museum), ISKCON Chowpatty (Radha Gopinath), Siddhivinayak, Mahalakshmi, Babulnath, Mumba Devi; Elephanta caves day trip. Was already on your Bucket List tab.</t>
+        </is>
+      </c>
+      <c r="J15" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K15" s="22" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="L15" s="22" t="inlineStr"/>
+      <c r="M15" s="22" t="inlineStr"/>
+      <c r="N15" s="12" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Kerala</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Kerala, India</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Temple + culture yatra</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Oct-Mar; Sabarimala season Nov-Jan</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Guruvayur Ekadasi (Nov-Dec); Thrissur Pooram (Apr-May)</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>None (domestic); Sabarimala needs virtual-queue booking</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>Guruvayur, Padmanabhaswamy (dress code), Sabarimala, Ambalappuzha, Aranmula, Chottanikkara; backwaters. Combine with Kanyakumari/Suchindram.</t>
+        </is>
+      </c>
+      <c r="J16" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K16" s="22" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="L16" s="22" t="inlineStr"/>
+      <c r="M16" s="22" t="inlineStr"/>
+      <c r="N16" s="12" t="n">
+        <v>46316</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:N113"/>
-  <conditionalFormatting sqref="K5:K113">
+  <autoFilter ref="A4:N116"/>
+  <conditionalFormatting sqref="K5:K116">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>"Done"</formula>
     </cfRule>
@@ -20473,10 +20653,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="K5:K113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K5:K116" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Idea,Researching,Planned,Booked,Done,Dropped"</formula1>
     </dataValidation>
-    <dataValidation sqref="J5:J113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J5:J116" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>